<commit_message>
Publish LiptovskyMikulas_2018_WC, Markkleeberg_2019_WC, Pau_2017_WCH, Pau_2020_WC
</commit_message>
<xml_diff>
--- a/events/Markkleeberg_2019_WC/Markkleeberg_2019_WC_start.xlsx
+++ b/events/Markkleeberg_2019_WC/Markkleeberg_2019_WC_start.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W534"/>
+  <dimension ref="A1:AC534"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -519,17 +519,47 @@
       </c>
       <c r="U1" t="inlineStr">
         <is>
+          <t>Name4</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>Name5</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>Name6</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
           <t>ICF_ID1</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>ICF_ID2</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>ICF_ID3</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>ICF_ID4</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
+          <t>ICF_ID5</t>
+        </is>
+      </c>
+      <c r="AC1" t="inlineStr">
+        <is>
+          <t>ICF_ID6</t>
         </is>
       </c>
     </row>
@@ -1171,7 +1201,7 @@
           <t>XU Yongzhao</t>
         </is>
       </c>
-      <c r="U14" t="inlineStr">
+      <c r="X14" t="inlineStr">
         <is>
           <t>69446</t>
         </is>
@@ -1229,7 +1259,7 @@
           <t>ZOU Weijian</t>
         </is>
       </c>
-      <c r="U15" t="inlineStr">
+      <c r="X15" t="inlineStr">
         <is>
           <t>94208</t>
         </is>
@@ -1287,7 +1317,7 @@
           <t>GIBBONS James</t>
         </is>
       </c>
-      <c r="U16" t="inlineStr">
+      <c r="X16" t="inlineStr">
         <is>
           <t>77314</t>
         </is>
@@ -1345,7 +1375,7 @@
           <t>LONG Tren</t>
         </is>
       </c>
-      <c r="U17" t="inlineStr">
+      <c r="X17" t="inlineStr">
         <is>
           <t>57124</t>
         </is>
@@ -1403,7 +1433,7 @@
           <t>TANIGUCHI Kazuya</t>
         </is>
       </c>
-      <c r="U18" t="inlineStr">
+      <c r="X18" t="inlineStr">
         <is>
           <t>39699</t>
         </is>
@@ -1461,7 +1491,7 @@
           <t>HUANG Fa</t>
         </is>
       </c>
-      <c r="U19" t="inlineStr">
+      <c r="X19" t="inlineStr">
         <is>
           <t>87703</t>
         </is>
@@ -1519,7 +1549,7 @@
           <t>POTOCNY Marcel</t>
         </is>
       </c>
-      <c r="U20" t="inlineStr">
+      <c r="X20" t="inlineStr">
         <is>
           <t>35235</t>
         </is>
@@ -1577,7 +1607,7 @@
           <t>CARVALHO Jose</t>
         </is>
       </c>
-      <c r="U21" t="inlineStr">
+      <c r="X21" t="inlineStr">
         <is>
           <t>35486</t>
         </is>
@@ -1635,7 +1665,7 @@
           <t>CONEY William</t>
         </is>
       </c>
-      <c r="U22" t="inlineStr">
+      <c r="X22" t="inlineStr">
         <is>
           <t>53138</t>
         </is>
@@ -1693,7 +1723,7 @@
           <t>CARTER Tristan</t>
         </is>
       </c>
-      <c r="U23" t="inlineStr">
+      <c r="X23" t="inlineStr">
         <is>
           <t>51890</t>
         </is>
@@ -1751,7 +1781,7 @@
           <t>COCHRANE Jake</t>
         </is>
       </c>
-      <c r="U24" t="inlineStr">
+      <c r="X24" t="inlineStr">
         <is>
           <t>60124</t>
         </is>
@@ -1862,7 +1892,7 @@
           <t>FERNANDEZ Luis</t>
         </is>
       </c>
-      <c r="U26" t="inlineStr">
+      <c r="X26" t="inlineStr">
         <is>
           <t>51851</t>
         </is>
@@ -1920,7 +1950,7 @@
           <t>HEGER Vojtech</t>
         </is>
       </c>
-      <c r="U27" t="inlineStr">
+      <c r="X27" t="inlineStr">
         <is>
           <t>68872</t>
         </is>
@@ -1978,7 +2008,7 @@
           <t>ROISIN Lucas</t>
         </is>
       </c>
-      <c r="U28" t="inlineStr">
+      <c r="X28" t="inlineStr">
         <is>
           <t>55580</t>
         </is>
@@ -2036,7 +2066,7 @@
           <t>CRAWFORD Brodie</t>
         </is>
       </c>
-      <c r="U29" t="inlineStr">
+      <c r="X29" t="inlineStr">
         <is>
           <t>38436</t>
         </is>
@@ -2094,7 +2124,7 @@
           <t>ABBOTT Thomas</t>
         </is>
       </c>
-      <c r="U30" t="inlineStr">
+      <c r="X30" t="inlineStr">
         <is>
           <t>36514</t>
         </is>
@@ -2152,7 +2182,7 @@
           <t>LOKKEN Zachary</t>
         </is>
       </c>
-      <c r="U31" t="inlineStr">
+      <c r="X31" t="inlineStr">
         <is>
           <t>35069</t>
         </is>
@@ -2210,7 +2240,7 @@
           <t>SZTUBA Igor</t>
         </is>
       </c>
-      <c r="U32" t="inlineStr">
+      <c r="X32" t="inlineStr">
         <is>
           <t>35087</t>
         </is>
@@ -2268,7 +2298,7 @@
           <t>TRUMMER Timo</t>
         </is>
       </c>
-      <c r="U33" t="inlineStr">
+      <c r="X33" t="inlineStr">
         <is>
           <t>41599</t>
         </is>
@@ -2326,7 +2356,7 @@
           <t>RAK Tomas</t>
         </is>
       </c>
-      <c r="U34" t="inlineStr">
+      <c r="X34" t="inlineStr">
         <is>
           <t>35056</t>
         </is>
@@ -2384,7 +2414,7 @@
           <t>BORROWS Ian</t>
         </is>
       </c>
-      <c r="U35" t="inlineStr">
+      <c r="X35" t="inlineStr">
         <is>
           <t>36534</t>
         </is>
@@ -2442,7 +2472,7 @@
           <t>KOECHLIN Thomas</t>
         </is>
       </c>
-      <c r="U36" t="inlineStr">
+      <c r="X36" t="inlineStr">
         <is>
           <t>35419</t>
         </is>
@@ -2500,7 +2530,7 @@
           <t>SZTUBA Kacper</t>
         </is>
       </c>
-      <c r="U37" t="inlineStr">
+      <c r="X37" t="inlineStr">
         <is>
           <t>53636</t>
         </is>
@@ -2558,7 +2588,7 @@
           <t>CIPRESSI Stefano</t>
         </is>
       </c>
-      <c r="U38" t="inlineStr">
+      <c r="X38" t="inlineStr">
         <is>
           <t>35495</t>
         </is>
@@ -2616,7 +2646,7 @@
           <t>GESTIN Nicolas</t>
         </is>
       </c>
-      <c r="U39" t="inlineStr">
+      <c r="X39" t="inlineStr">
         <is>
           <t>71961</t>
         </is>
@@ -2674,7 +2704,7 @@
           <t>TRAVE Miquel</t>
         </is>
       </c>
-      <c r="U40" t="inlineStr">
+      <c r="X40" t="inlineStr">
         <is>
           <t>68998</t>
         </is>
@@ -2732,7 +2762,7 @@
           <t>ELOSEGI Ander</t>
         </is>
       </c>
-      <c r="U41" t="inlineStr">
+      <c r="X41" t="inlineStr">
         <is>
           <t>35785</t>
         </is>
@@ -2790,7 +2820,7 @@
           <t>IVALDI Raffaello</t>
         </is>
       </c>
-      <c r="U42" t="inlineStr">
+      <c r="X42" t="inlineStr">
         <is>
           <t>35227</t>
         </is>
@@ -2848,7 +2878,7 @@
           <t>EICHFELD Casey</t>
         </is>
       </c>
-      <c r="U43" t="inlineStr">
+      <c r="X43" t="inlineStr">
         <is>
           <t>35067</t>
         </is>
@@ -2906,7 +2936,7 @@
           <t>ROHAN Lukas</t>
         </is>
       </c>
-      <c r="U44" t="inlineStr">
+      <c r="X44" t="inlineStr">
         <is>
           <t>36114</t>
         </is>
@@ -2964,7 +2994,7 @@
           <t>HEDWIG Grzegorz</t>
         </is>
       </c>
-      <c r="U45" t="inlineStr">
+      <c r="X45" t="inlineStr">
         <is>
           <t>35465</t>
         </is>
@@ -3022,7 +3052,7 @@
           <t>BERCIC Anze</t>
         </is>
       </c>
-      <c r="U46" t="inlineStr">
+      <c r="X46" t="inlineStr">
         <is>
           <t>36253</t>
         </is>
@@ -3080,7 +3110,7 @@
           <t>COLAZINGARI Roberto</t>
         </is>
       </c>
-      <c r="U47" t="inlineStr">
+      <c r="X47" t="inlineStr">
         <is>
           <t>35223</t>
         </is>
@@ -3138,7 +3168,7 @@
           <t>GARGAUD CHANUT Denis</t>
         </is>
       </c>
-      <c r="U48" t="inlineStr">
+      <c r="X48" t="inlineStr">
         <is>
           <t>35177</t>
         </is>
@@ -3196,7 +3226,7 @@
           <t>MARTIKAN Michal</t>
         </is>
       </c>
-      <c r="U49" t="inlineStr">
+      <c r="X49" t="inlineStr">
         <is>
           <t>35365</t>
         </is>
@@ -3254,7 +3284,7 @@
           <t>BENUS Matej</t>
         </is>
       </c>
-      <c r="U50" t="inlineStr">
+      <c r="X50" t="inlineStr">
         <is>
           <t>35353</t>
         </is>
@@ -3312,7 +3342,7 @@
           <t>SAVSEK Benjamin</t>
         </is>
       </c>
-      <c r="U51" t="inlineStr">
+      <c r="X51" t="inlineStr">
         <is>
           <t>36218</t>
         </is>
@@ -3370,7 +3400,7 @@
           <t>BOZIC Luka</t>
         </is>
       </c>
-      <c r="U52" t="inlineStr">
+      <c r="X52" t="inlineStr">
         <is>
           <t>36269</t>
         </is>
@@ -3428,7 +3458,7 @@
           <t>ANTON Franz</t>
         </is>
       </c>
-      <c r="U53" t="inlineStr">
+      <c r="X53" t="inlineStr">
         <is>
           <t>35137</t>
         </is>
@@ -3486,7 +3516,7 @@
           <t>SLAFKOVSKY Alexander</t>
         </is>
       </c>
-      <c r="U54" t="inlineStr">
+      <c r="X54" t="inlineStr">
         <is>
           <t>35129</t>
         </is>
@@ -3544,7 +3574,7 @@
           <t>TASIADIS Sideris</t>
         </is>
       </c>
-      <c r="U55" t="inlineStr">
+      <c r="X55" t="inlineStr">
         <is>
           <t>35135</t>
         </is>
@@ -3602,7 +3632,7 @@
           <t>STACH Aleksandra</t>
         </is>
       </c>
-      <c r="U56" t="inlineStr">
+      <c r="X56" t="inlineStr">
         <is>
           <t>61261</t>
         </is>
@@ -3660,7 +3690,7 @@
           <t>SETCHELL Nikita</t>
         </is>
       </c>
-      <c r="U57" t="inlineStr">
+      <c r="X57" t="inlineStr">
         <is>
           <t>86250</t>
         </is>
@@ -3718,7 +3748,7 @@
           <t>XU Yanru</t>
         </is>
       </c>
-      <c r="U58" t="inlineStr">
+      <c r="X58" t="inlineStr">
         <is>
           <t>63801</t>
         </is>
@@ -3776,7 +3806,7 @@
           <t>KRIESINGER Janina</t>
         </is>
       </c>
-      <c r="U59" t="inlineStr">
+      <c r="X59" t="inlineStr">
         <is>
           <t>93682</t>
         </is>
@@ -3834,7 +3864,7 @@
           <t>SORRIBES Laia</t>
         </is>
       </c>
-      <c r="U60" t="inlineStr">
+      <c r="X60" t="inlineStr">
         <is>
           <t>68822</t>
         </is>
@@ -3892,7 +3922,7 @@
           <t>LEIBFARTH Evy</t>
         </is>
       </c>
-      <c r="U61" t="inlineStr">
+      <c r="X61" t="inlineStr">
         <is>
           <t>83538</t>
         </is>
@@ -3950,7 +3980,7 @@
           <t>KAIFUCHI Moe</t>
         </is>
       </c>
-      <c r="U62" t="inlineStr">
+      <c r="X62" t="inlineStr">
         <is>
           <t>36483</t>
         </is>
@@ -4008,7 +4038,7 @@
           <t>MARX Alena</t>
         </is>
       </c>
-      <c r="U63" t="inlineStr">
+      <c r="X63" t="inlineStr">
         <is>
           <t>68844</t>
         </is>
@@ -4066,7 +4096,7 @@
           <t>MALAGUTI Francesca</t>
         </is>
       </c>
-      <c r="U64" t="inlineStr">
+      <c r="X64" t="inlineStr">
         <is>
           <t>77362</t>
         </is>
@@ -4124,7 +4154,7 @@
           <t>BRAENDLE Naemi</t>
         </is>
       </c>
-      <c r="U65" t="inlineStr">
+      <c r="X65" t="inlineStr">
         <is>
           <t>68845</t>
         </is>
@@ -4182,7 +4212,7 @@
           <t>MITASIKOVA Monika</t>
         </is>
       </c>
-      <c r="U66" t="inlineStr">
+      <c r="X66" t="inlineStr">
         <is>
           <t>75445</t>
         </is>
@@ -4240,7 +4270,7 @@
           <t>MASLEN Amber</t>
         </is>
       </c>
-      <c r="U67" t="inlineStr">
+      <c r="X67" t="inlineStr">
         <is>
           <t>53074</t>
         </is>
@@ -4298,7 +4328,7 @@
           <t>HOCEVAR Eva Alina</t>
         </is>
       </c>
-      <c r="U68" t="inlineStr">
+      <c r="X68" t="inlineStr">
         <is>
           <t>75533</t>
         </is>
@@ -4356,7 +4386,7 @@
           <t>LEENDERS Claudia</t>
         </is>
       </c>
-      <c r="U69" t="inlineStr">
+      <c r="X69" t="inlineStr">
         <is>
           <t>35331</t>
         </is>
@@ -4414,7 +4444,7 @@
           <t>TEUNISSEN Lena</t>
         </is>
       </c>
-      <c r="U70" t="inlineStr">
+      <c r="X70" t="inlineStr">
         <is>
           <t>35344</t>
         </is>
@@ -4472,7 +4502,7 @@
           <t>NEE Ashley</t>
         </is>
       </c>
-      <c r="U71" t="inlineStr">
+      <c r="X71" t="inlineStr">
         <is>
           <t>36363</t>
         </is>
@@ -4530,7 +4560,7 @@
           <t>HAMER-EVANS Megan</t>
         </is>
       </c>
-      <c r="U72" t="inlineStr">
+      <c r="X72" t="inlineStr">
         <is>
           <t>55138</t>
         </is>
@@ -4588,7 +4618,7 @@
           <t>APEL Elena</t>
         </is>
       </c>
-      <c r="U73" t="inlineStr">
+      <c r="X73" t="inlineStr">
         <is>
           <t>51837</t>
         </is>
@@ -4646,7 +4676,7 @@
           <t>FOX Noemie</t>
         </is>
       </c>
-      <c r="U74" t="inlineStr">
+      <c r="X74" t="inlineStr">
         <is>
           <t>44812</t>
         </is>
@@ -4704,7 +4734,7 @@
           <t>WERATSCHNIG Nina</t>
         </is>
       </c>
-      <c r="U75" t="inlineStr">
+      <c r="X75" t="inlineStr">
         <is>
           <t>41614</t>
         </is>
@@ -4762,7 +4792,7 @@
           <t>DORIA VILARRUBLA Monica</t>
         </is>
       </c>
-      <c r="U76" t="inlineStr">
+      <c r="X76" t="inlineStr">
         <is>
           <t>53051</t>
         </is>
@@ -4820,7 +4850,7 @@
           <t>NOVAK Ajda</t>
         </is>
       </c>
-      <c r="U77" t="inlineStr">
+      <c r="X77" t="inlineStr">
         <is>
           <t>39079</t>
         </is>
@@ -4878,7 +4908,7 @@
           <t>LI Tong</t>
         </is>
       </c>
-      <c r="U78" t="inlineStr">
+      <c r="X78" t="inlineStr">
         <is>
           <t>52023</t>
         </is>
@@ -4936,7 +4966,7 @@
           <t>KALISKA Elena</t>
         </is>
       </c>
-      <c r="U79" t="inlineStr">
+      <c r="X79" t="inlineStr">
         <is>
           <t>35366</t>
         </is>
@@ -4994,7 +5024,7 @@
           <t>MINTALOVA Eliska</t>
         </is>
       </c>
-      <c r="U80" t="inlineStr">
+      <c r="X80" t="inlineStr">
         <is>
           <t>56169</t>
         </is>
@@ -5052,7 +5082,7 @@
           <t>ECKHARDT Kate</t>
         </is>
       </c>
-      <c r="U81" t="inlineStr">
+      <c r="X81" t="inlineStr">
         <is>
           <t>44815</t>
         </is>
@@ -5110,7 +5140,7 @@
           <t>HILGERTOVA Amalie</t>
         </is>
       </c>
-      <c r="U82" t="inlineStr">
+      <c r="X82" t="inlineStr">
         <is>
           <t>36113</t>
         </is>
@@ -5168,7 +5198,7 @@
           <t>WEGMAN Martina</t>
         </is>
       </c>
-      <c r="U83" t="inlineStr">
+      <c r="X83" t="inlineStr">
         <is>
           <t>35345</t>
         </is>
@@ -5226,7 +5256,7 @@
           <t>PACIERPNIK Natalia</t>
         </is>
       </c>
-      <c r="U84" t="inlineStr">
+      <c r="X84" t="inlineStr">
         <is>
           <t>35077</t>
         </is>
@@ -5284,7 +5314,7 @@
           <t>DUKATOVA Jana</t>
         </is>
       </c>
-      <c r="U85" t="inlineStr">
+      <c r="X85" t="inlineStr">
         <is>
           <t>35354</t>
         </is>
@@ -5342,7 +5372,7 @@
           <t>ZWOLINSKA Klaudia</t>
         </is>
       </c>
-      <c r="U86" t="inlineStr">
+      <c r="X86" t="inlineStr">
         <is>
           <t>42027</t>
         </is>
@@ -5400,7 +5430,7 @@
           <t>LAFONT Marie-Zelia</t>
         </is>
       </c>
-      <c r="U87" t="inlineStr">
+      <c r="X87" t="inlineStr">
         <is>
           <t>35374</t>
         </is>
@@ -5458,7 +5488,7 @@
           <t>BAUDU Lucie</t>
         </is>
       </c>
-      <c r="U88" t="inlineStr">
+      <c r="X88" t="inlineStr">
         <is>
           <t>35669</t>
         </is>
@@ -5516,7 +5546,7 @@
           <t>VOJTOVA Veronika</t>
         </is>
       </c>
-      <c r="U89" t="inlineStr">
+      <c r="X89" t="inlineStr">
         <is>
           <t>35945</t>
         </is>
@@ -5574,7 +5604,7 @@
           <t>SCHORNBERG Jasmin</t>
         </is>
       </c>
-      <c r="U90" t="inlineStr">
+      <c r="X90" t="inlineStr">
         <is>
           <t>35206</t>
         </is>
@@ -5632,7 +5662,7 @@
           <t>SATILA Ana</t>
         </is>
       </c>
-      <c r="U91" t="inlineStr">
+      <c r="X91" t="inlineStr">
         <is>
           <t>35327</t>
         </is>
@@ -5690,7 +5720,7 @@
           <t>WOLFFHARDT Viktoria</t>
         </is>
       </c>
-      <c r="U92" t="inlineStr">
+      <c r="X92" t="inlineStr">
         <is>
           <t>35303</t>
         </is>
@@ -5748,7 +5778,7 @@
           <t>KUDEJOVA Katerina</t>
         </is>
       </c>
-      <c r="U93" t="inlineStr">
+      <c r="X93" t="inlineStr">
         <is>
           <t>35034</t>
         </is>
@@ -5806,7 +5836,7 @@
           <t>TERCELJ Eva</t>
         </is>
       </c>
-      <c r="U94" t="inlineStr">
+      <c r="X94" t="inlineStr">
         <is>
           <t>36263</t>
         </is>
@@ -5864,7 +5894,7 @@
           <t>PRIGENT Camille</t>
         </is>
       </c>
-      <c r="U95" t="inlineStr">
+      <c r="X95" t="inlineStr">
         <is>
           <t>41566</t>
         </is>
@@ -5922,7 +5952,7 @@
           <t>HORN Stefanie</t>
         </is>
       </c>
-      <c r="U96" t="inlineStr">
+      <c r="X96" t="inlineStr">
         <is>
           <t>38417</t>
         </is>
@@ -5980,7 +6010,7 @@
           <t>CHOURRAUT Maialen</t>
         </is>
       </c>
-      <c r="U97" t="inlineStr">
+      <c r="X97" t="inlineStr">
         <is>
           <t>35787</t>
         </is>
@@ -6038,7 +6068,7 @@
           <t>KUHNLE Corinna</t>
         </is>
       </c>
-      <c r="U98" t="inlineStr">
+      <c r="X98" t="inlineStr">
         <is>
           <t>35282</t>
         </is>
@@ -6096,7 +6126,7 @@
           <t>FUNK Ricarda</t>
         </is>
       </c>
-      <c r="U99" t="inlineStr">
+      <c r="X99" t="inlineStr">
         <is>
           <t>35122</t>
         </is>
@@ -6154,7 +6184,7 @@
           <t>FOX Jessica</t>
         </is>
       </c>
-      <c r="U100" t="inlineStr">
+      <c r="X100" t="inlineStr">
         <is>
           <t>36526</t>
         </is>
@@ -6212,7 +6242,7 @@
           <t>XU Yongzhao</t>
         </is>
       </c>
-      <c r="U101" t="inlineStr">
+      <c r="X101" t="inlineStr">
         <is>
           <t>69446</t>
         </is>
@@ -6270,7 +6300,7 @@
           <t>ZOU Weijian</t>
         </is>
       </c>
-      <c r="U102" t="inlineStr">
+      <c r="X102" t="inlineStr">
         <is>
           <t>94208</t>
         </is>
@@ -6328,7 +6358,7 @@
           <t>GIBBONS James</t>
         </is>
       </c>
-      <c r="U103" t="inlineStr">
+      <c r="X103" t="inlineStr">
         <is>
           <t>77314</t>
         </is>
@@ -6386,7 +6416,7 @@
           <t>LONG Tren</t>
         </is>
       </c>
-      <c r="U104" t="inlineStr">
+      <c r="X104" t="inlineStr">
         <is>
           <t>57124</t>
         </is>
@@ -6444,7 +6474,7 @@
           <t>TANIGUCHI Kazuya</t>
         </is>
       </c>
-      <c r="U105" t="inlineStr">
+      <c r="X105" t="inlineStr">
         <is>
           <t>39699</t>
         </is>
@@ -6502,7 +6532,7 @@
           <t>HUANG Fa</t>
         </is>
       </c>
-      <c r="U106" t="inlineStr">
+      <c r="X106" t="inlineStr">
         <is>
           <t>87703</t>
         </is>
@@ -6560,7 +6590,7 @@
           <t>POTOCNY Marcel</t>
         </is>
       </c>
-      <c r="U107" t="inlineStr">
+      <c r="X107" t="inlineStr">
         <is>
           <t>35235</t>
         </is>
@@ -6618,7 +6648,7 @@
           <t>CARVALHO Jose</t>
         </is>
       </c>
-      <c r="U108" t="inlineStr">
+      <c r="X108" t="inlineStr">
         <is>
           <t>35486</t>
         </is>
@@ -6676,7 +6706,7 @@
           <t>CONEY William</t>
         </is>
       </c>
-      <c r="U109" t="inlineStr">
+      <c r="X109" t="inlineStr">
         <is>
           <t>53138</t>
         </is>
@@ -6734,7 +6764,7 @@
           <t>CARTER Tristan</t>
         </is>
       </c>
-      <c r="U110" t="inlineStr">
+      <c r="X110" t="inlineStr">
         <is>
           <t>51890</t>
         </is>
@@ -6792,7 +6822,7 @@
           <t>COCHRANE Jake</t>
         </is>
       </c>
-      <c r="U111" t="inlineStr">
+      <c r="X111" t="inlineStr">
         <is>
           <t>60124</t>
         </is>
@@ -6903,7 +6933,7 @@
           <t>FERNANDEZ Luis</t>
         </is>
       </c>
-      <c r="U113" t="inlineStr">
+      <c r="X113" t="inlineStr">
         <is>
           <t>51851</t>
         </is>
@@ -6961,7 +6991,7 @@
           <t>ROISIN Lucas</t>
         </is>
       </c>
-      <c r="U114" t="inlineStr">
+      <c r="X114" t="inlineStr">
         <is>
           <t>55580</t>
         </is>
@@ -7019,7 +7049,7 @@
           <t>CRAWFORD Brodie</t>
         </is>
       </c>
-      <c r="U115" t="inlineStr">
+      <c r="X115" t="inlineStr">
         <is>
           <t>38436</t>
         </is>
@@ -7077,7 +7107,7 @@
           <t>SZTUBA Igor</t>
         </is>
       </c>
-      <c r="U116" t="inlineStr">
+      <c r="X116" t="inlineStr">
         <is>
           <t>35087</t>
         </is>
@@ -7135,7 +7165,7 @@
           <t>TRUMMER Timo</t>
         </is>
       </c>
-      <c r="U117" t="inlineStr">
+      <c r="X117" t="inlineStr">
         <is>
           <t>41599</t>
         </is>
@@ -7193,7 +7223,7 @@
           <t>BORROWS Ian</t>
         </is>
       </c>
-      <c r="U118" t="inlineStr">
+      <c r="X118" t="inlineStr">
         <is>
           <t>36534</t>
         </is>
@@ -7251,7 +7281,7 @@
           <t>KOECHLIN Thomas</t>
         </is>
       </c>
-      <c r="U119" t="inlineStr">
+      <c r="X119" t="inlineStr">
         <is>
           <t>35419</t>
         </is>
@@ -7309,7 +7339,7 @@
           <t>GESTIN Nicolas</t>
         </is>
       </c>
-      <c r="U120" t="inlineStr">
+      <c r="X120" t="inlineStr">
         <is>
           <t>71961</t>
         </is>
@@ -7367,7 +7397,7 @@
           <t>EICHFELD Casey</t>
         </is>
       </c>
-      <c r="U121" t="inlineStr">
+      <c r="X121" t="inlineStr">
         <is>
           <t>35067</t>
         </is>
@@ -7425,7 +7455,7 @@
           <t>HEDWIG Grzegorz</t>
         </is>
       </c>
-      <c r="U122" t="inlineStr">
+      <c r="X122" t="inlineStr">
         <is>
           <t>35465</t>
         </is>
@@ -7483,7 +7513,7 @@
           <t>STACH Aleksandra</t>
         </is>
       </c>
-      <c r="U123" t="inlineStr">
+      <c r="X123" t="inlineStr">
         <is>
           <t>61261</t>
         </is>
@@ -7541,7 +7571,7 @@
           <t>SETCHELL Nikita</t>
         </is>
       </c>
-      <c r="U124" t="inlineStr">
+      <c r="X124" t="inlineStr">
         <is>
           <t>86250</t>
         </is>
@@ -7599,7 +7629,7 @@
           <t>XU Yanru</t>
         </is>
       </c>
-      <c r="U125" t="inlineStr">
+      <c r="X125" t="inlineStr">
         <is>
           <t>63801</t>
         </is>
@@ -7657,7 +7687,7 @@
           <t>KRIESINGER Janina</t>
         </is>
       </c>
-      <c r="U126" t="inlineStr">
+      <c r="X126" t="inlineStr">
         <is>
           <t>93682</t>
         </is>
@@ -7715,7 +7745,7 @@
           <t>SORRIBES Laia</t>
         </is>
       </c>
-      <c r="U127" t="inlineStr">
+      <c r="X127" t="inlineStr">
         <is>
           <t>68822</t>
         </is>
@@ -7773,7 +7803,7 @@
           <t>KAIFUCHI Moe</t>
         </is>
       </c>
-      <c r="U128" t="inlineStr">
+      <c r="X128" t="inlineStr">
         <is>
           <t>36483</t>
         </is>
@@ -7831,7 +7861,7 @@
           <t>MARX Alena</t>
         </is>
       </c>
-      <c r="U129" t="inlineStr">
+      <c r="X129" t="inlineStr">
         <is>
           <t>68844</t>
         </is>
@@ -7889,7 +7919,7 @@
           <t>MALAGUTI Francesca</t>
         </is>
       </c>
-      <c r="U130" t="inlineStr">
+      <c r="X130" t="inlineStr">
         <is>
           <t>77362</t>
         </is>
@@ -7947,7 +7977,7 @@
           <t>BRAENDLE Naemi</t>
         </is>
       </c>
-      <c r="U131" t="inlineStr">
+      <c r="X131" t="inlineStr">
         <is>
           <t>68845</t>
         </is>
@@ -8005,7 +8035,7 @@
           <t>MITASIKOVA Monika</t>
         </is>
       </c>
-      <c r="U132" t="inlineStr">
+      <c r="X132" t="inlineStr">
         <is>
           <t>75445</t>
         </is>
@@ -8063,7 +8093,7 @@
           <t>MASLEN Amber</t>
         </is>
       </c>
-      <c r="U133" t="inlineStr">
+      <c r="X133" t="inlineStr">
         <is>
           <t>53074</t>
         </is>
@@ -8121,7 +8151,7 @@
           <t>HOCEVAR Eva Alina</t>
         </is>
       </c>
-      <c r="U134" t="inlineStr">
+      <c r="X134" t="inlineStr">
         <is>
           <t>75533</t>
         </is>
@@ -8179,7 +8209,7 @@
           <t>TEUNISSEN Lena</t>
         </is>
       </c>
-      <c r="U135" t="inlineStr">
+      <c r="X135" t="inlineStr">
         <is>
           <t>35344</t>
         </is>
@@ -8237,7 +8267,7 @@
           <t>NEE Ashley</t>
         </is>
       </c>
-      <c r="U136" t="inlineStr">
+      <c r="X136" t="inlineStr">
         <is>
           <t>36363</t>
         </is>
@@ -8295,7 +8325,7 @@
           <t>FOX Noemie</t>
         </is>
       </c>
-      <c r="U137" t="inlineStr">
+      <c r="X137" t="inlineStr">
         <is>
           <t>44812</t>
         </is>
@@ -8353,7 +8383,7 @@
           <t>WERATSCHNIG Nina</t>
         </is>
       </c>
-      <c r="U138" t="inlineStr">
+      <c r="X138" t="inlineStr">
         <is>
           <t>41614</t>
         </is>
@@ -8411,7 +8441,7 @@
           <t>DORIA VILARRUBLA Monica</t>
         </is>
       </c>
-      <c r="U139" t="inlineStr">
+      <c r="X139" t="inlineStr">
         <is>
           <t>53051</t>
         </is>
@@ -8469,7 +8499,7 @@
           <t>NOVAK Ajda</t>
         </is>
       </c>
-      <c r="U140" t="inlineStr">
+      <c r="X140" t="inlineStr">
         <is>
           <t>39079</t>
         </is>
@@ -8527,7 +8557,7 @@
           <t>LI Tong</t>
         </is>
       </c>
-      <c r="U141" t="inlineStr">
+      <c r="X141" t="inlineStr">
         <is>
           <t>52023</t>
         </is>
@@ -8585,7 +8615,7 @@
           <t>MINTALOVA Eliska</t>
         </is>
       </c>
-      <c r="U142" t="inlineStr">
+      <c r="X142" t="inlineStr">
         <is>
           <t>56169</t>
         </is>
@@ -8643,7 +8673,7 @@
           <t>ECKHARDT Kate</t>
         </is>
       </c>
-      <c r="U143" t="inlineStr">
+      <c r="X143" t="inlineStr">
         <is>
           <t>44815</t>
         </is>
@@ -8701,7 +8731,7 @@
           <t>HILGERTOVA Amalie</t>
         </is>
       </c>
-      <c r="U144" t="inlineStr">
+      <c r="X144" t="inlineStr">
         <is>
           <t>36113</t>
         </is>
@@ -8759,7 +8789,7 @@
           <t>WEGMAN Martina</t>
         </is>
       </c>
-      <c r="U145" t="inlineStr">
+      <c r="X145" t="inlineStr">
         <is>
           <t>35345</t>
         </is>
@@ -8817,7 +8847,7 @@
           <t>DUKATOVA Jana</t>
         </is>
       </c>
-      <c r="U146" t="inlineStr">
+      <c r="X146" t="inlineStr">
         <is>
           <t>35354</t>
         </is>
@@ -8875,7 +8905,7 @@
           <t>VOJTOVA Veronika</t>
         </is>
       </c>
-      <c r="U147" t="inlineStr">
+      <c r="X147" t="inlineStr">
         <is>
           <t>35945</t>
         </is>
@@ -9145,7 +9175,7 @@
           <t>ZWOLINSKA Klaudia</t>
         </is>
       </c>
-      <c r="U152" t="inlineStr">
+      <c r="X152" t="inlineStr">
         <is>
           <t>42027</t>
         </is>
@@ -9203,7 +9233,7 @@
           <t>YU Cuishan</t>
         </is>
       </c>
-      <c r="U153" t="inlineStr">
+      <c r="X153" t="inlineStr">
         <is>
           <t>75380</t>
         </is>
@@ -9261,7 +9291,7 @@
           <t>LAMEIRO Ainhoa</t>
         </is>
       </c>
-      <c r="U154" t="inlineStr">
+      <c r="X154" t="inlineStr">
         <is>
           <t>69042</t>
         </is>
@@ -9319,7 +9349,7 @@
           <t>TENG Qianqian</t>
         </is>
       </c>
-      <c r="U155" t="inlineStr">
+      <c r="X155" t="inlineStr">
         <is>
           <t>94209</t>
         </is>
@@ -9377,7 +9407,7 @@
           <t>LEIBFARTH Evy</t>
         </is>
       </c>
-      <c r="U156" t="inlineStr">
+      <c r="X156" t="inlineStr">
         <is>
           <t>83538</t>
         </is>
@@ -9435,7 +9465,7 @@
           <t>MICOZZI Elena</t>
         </is>
       </c>
-      <c r="U157" t="inlineStr">
+      <c r="X157" t="inlineStr">
         <is>
           <t>84644</t>
         </is>
@@ -9493,7 +9523,7 @@
           <t>MARX Alena</t>
         </is>
       </c>
-      <c r="U158" t="inlineStr">
+      <c r="X158" t="inlineStr">
         <is>
           <t>68844</t>
         </is>
@@ -9551,7 +9581,7 @@
           <t>MILLER Ellis</t>
         </is>
       </c>
-      <c r="U159" t="inlineStr">
+      <c r="X159" t="inlineStr">
         <is>
           <t>75828</t>
         </is>
@@ -9609,7 +9639,7 @@
           <t>SPICER Phoebe</t>
         </is>
       </c>
-      <c r="U160" t="inlineStr">
+      <c r="X160" t="inlineStr">
         <is>
           <t>75827</t>
         </is>
@@ -9667,7 +9697,7 @@
           <t>NOVAK Lea</t>
         </is>
       </c>
-      <c r="U161" t="inlineStr">
+      <c r="X161" t="inlineStr">
         <is>
           <t>60323</t>
         </is>
@@ -9725,7 +9755,7 @@
           <t>YAGI Airi</t>
         </is>
       </c>
-      <c r="U162" t="inlineStr">
+      <c r="X162" t="inlineStr">
         <is>
           <t>37756</t>
         </is>
@@ -9783,7 +9813,7 @@
           <t>BERTONCELLI Marta</t>
         </is>
       </c>
-      <c r="U163" t="inlineStr">
+      <c r="X163" t="inlineStr">
         <is>
           <t>71982</t>
         </is>
@@ -9841,7 +9871,7 @@
           <t>STACH Aleksandra</t>
         </is>
       </c>
-      <c r="U164" t="inlineStr">
+      <c r="X164" t="inlineStr">
         <is>
           <t>61261</t>
         </is>
@@ -9899,7 +9929,7 @@
           <t>SCHORNBERG Jasmin</t>
         </is>
       </c>
-      <c r="U165" t="inlineStr">
+      <c r="X165" t="inlineStr">
         <is>
           <t>35206</t>
         </is>
@@ -9957,7 +9987,7 @@
           <t>LUKNAROVA Emanuela</t>
         </is>
       </c>
-      <c r="U166" t="inlineStr">
+      <c r="X166" t="inlineStr">
         <is>
           <t>76973</t>
         </is>
@@ -10015,7 +10045,7 @@
           <t>BREGAZZI Ella</t>
         </is>
       </c>
-      <c r="U167" t="inlineStr">
+      <c r="X167" t="inlineStr">
         <is>
           <t>41598</t>
         </is>
@@ -10073,7 +10103,7 @@
           <t>DONNELLY Sage</t>
         </is>
       </c>
-      <c r="U168" t="inlineStr">
+      <c r="X168" t="inlineStr">
         <is>
           <t>60119</t>
         </is>
@@ -10131,7 +10161,7 @@
           <t>RIHOVA Eva</t>
         </is>
       </c>
-      <c r="U169" t="inlineStr">
+      <c r="X169" t="inlineStr">
         <is>
           <t>51791</t>
         </is>
@@ -10189,7 +10219,7 @@
           <t>HAVLICKOVA Katerina</t>
         </is>
       </c>
-      <c r="U170" t="inlineStr">
+      <c r="X170" t="inlineStr">
         <is>
           <t>35048</t>
         </is>
@@ -10247,7 +10277,7 @@
           <t>HOCEVAR Eva Alina</t>
         </is>
       </c>
-      <c r="U171" t="inlineStr">
+      <c r="X171" t="inlineStr">
         <is>
           <t>75533</t>
         </is>
@@ -10305,7 +10335,7 @@
           <t>FORROW Bethan</t>
         </is>
       </c>
-      <c r="U172" t="inlineStr">
+      <c r="X172" t="inlineStr">
         <is>
           <t>69065</t>
         </is>
@@ -10363,7 +10393,7 @@
           <t>ECKHARDT Kate</t>
         </is>
       </c>
-      <c r="U173" t="inlineStr">
+      <c r="X173" t="inlineStr">
         <is>
           <t>44815</t>
         </is>
@@ -10421,7 +10451,7 @@
           <t>CHEN Shi</t>
         </is>
       </c>
-      <c r="U174" t="inlineStr">
+      <c r="X174" t="inlineStr">
         <is>
           <t>52027</t>
         </is>
@@ -10479,7 +10509,7 @@
           <t>APEL Elena</t>
         </is>
       </c>
-      <c r="U175" t="inlineStr">
+      <c r="X175" t="inlineStr">
         <is>
           <t>51837</t>
         </is>
@@ -10537,7 +10567,7 @@
           <t>DELASSUS Marjorie</t>
         </is>
       </c>
-      <c r="U176" t="inlineStr">
+      <c r="X176" t="inlineStr">
         <is>
           <t>71964</t>
         </is>
@@ -10595,7 +10625,7 @@
           <t>KOZOROG Alja</t>
         </is>
       </c>
-      <c r="U177" t="inlineStr">
+      <c r="X177" t="inlineStr">
         <is>
           <t>39986</t>
         </is>
@@ -10653,7 +10683,7 @@
           <t>SKACHOVA Monika</t>
         </is>
       </c>
-      <c r="U178" t="inlineStr">
+      <c r="X178" t="inlineStr">
         <is>
           <t>53078</t>
         </is>
@@ -10711,7 +10741,7 @@
           <t>STANOVSKA Sona</t>
         </is>
       </c>
-      <c r="U179" t="inlineStr">
+      <c r="X179" t="inlineStr">
         <is>
           <t>51647</t>
         </is>
@@ -10769,7 +10799,7 @@
           <t>OLAZABAL Klara</t>
         </is>
       </c>
-      <c r="U180" t="inlineStr">
+      <c r="X180" t="inlineStr">
         <is>
           <t>43985</t>
         </is>
@@ -10827,7 +10857,7 @@
           <t>DORIA VILARRUBLA Monica</t>
         </is>
       </c>
-      <c r="U181" t="inlineStr">
+      <c r="X181" t="inlineStr">
         <is>
           <t>53051</t>
         </is>
@@ -10885,7 +10915,7 @@
           <t>BAUDU Lucie</t>
         </is>
       </c>
-      <c r="U182" t="inlineStr">
+      <c r="X182" t="inlineStr">
         <is>
           <t>35669</t>
         </is>
@@ -10943,7 +10973,7 @@
           <t>FOX Noemie</t>
         </is>
       </c>
-      <c r="U183" t="inlineStr">
+      <c r="X183" t="inlineStr">
         <is>
           <t>44812</t>
         </is>
@@ -11001,7 +11031,7 @@
           <t>HERZOG Andrea</t>
         </is>
       </c>
-      <c r="U184" t="inlineStr">
+      <c r="X184" t="inlineStr">
         <is>
           <t>55099</t>
         </is>
@@ -11059,7 +11089,7 @@
           <t>VILARRUBLA Nuria</t>
         </is>
       </c>
-      <c r="U185" t="inlineStr">
+      <c r="X185" t="inlineStr">
         <is>
           <t>35746</t>
         </is>
@@ -11117,7 +11147,7 @@
           <t>FISEROVA Tereza</t>
         </is>
       </c>
-      <c r="U186" t="inlineStr">
+      <c r="X186" t="inlineStr">
         <is>
           <t>42016</t>
         </is>
@@ -11175,7 +11205,7 @@
           <t>WERATSCHNIG Nadine</t>
         </is>
       </c>
-      <c r="U187" t="inlineStr">
+      <c r="X187" t="inlineStr">
         <is>
           <t>41613</t>
         </is>
@@ -11233,7 +11263,7 @@
           <t>WOLFFHARDT Viktoria</t>
         </is>
       </c>
-      <c r="U188" t="inlineStr">
+      <c r="X188" t="inlineStr">
         <is>
           <t>35303</t>
         </is>
@@ -11291,7 +11321,7 @@
           <t>SATILA Ana</t>
         </is>
       </c>
-      <c r="U189" t="inlineStr">
+      <c r="X189" t="inlineStr">
         <is>
           <t>35327</t>
         </is>
@@ -11349,7 +11379,7 @@
           <t>FOX Jessica</t>
         </is>
       </c>
-      <c r="U190" t="inlineStr">
+      <c r="X190" t="inlineStr">
         <is>
           <t>36526</t>
         </is>
@@ -11407,7 +11437,7 @@
           <t>CHEN Tianlu</t>
         </is>
       </c>
-      <c r="U191" t="inlineStr">
+      <c r="X191" t="inlineStr">
         <is>
           <t>84748</t>
         </is>
@@ -11465,7 +11495,7 @@
           <t>CELMINS Ritvars</t>
         </is>
       </c>
-      <c r="U192" t="inlineStr">
+      <c r="X192" t="inlineStr">
         <is>
           <t>35182</t>
         </is>
@@ -11523,7 +11553,7 @@
           <t>KOJIMA Daichi</t>
         </is>
       </c>
-      <c r="U193" t="inlineStr">
+      <c r="X193" t="inlineStr">
         <is>
           <t>42255</t>
         </is>
@@ -11581,7 +11611,7 @@
           <t>SWETNAM Huw</t>
         </is>
       </c>
-      <c r="U194" t="inlineStr">
+      <c r="X194" t="inlineStr">
         <is>
           <t>35652</t>
         </is>
@@ -11639,7 +11669,7 @@
           <t>MUTO Yusuke</t>
         </is>
       </c>
-      <c r="U195" t="inlineStr">
+      <c r="X195" t="inlineStr">
         <is>
           <t>71820</t>
         </is>
@@ -11697,7 +11727,7 @@
           <t>TANAKA Yuuki</t>
         </is>
       </c>
-      <c r="U196" t="inlineStr">
+      <c r="X196" t="inlineStr">
         <is>
           <t>75422</t>
         </is>
@@ -11755,7 +11785,7 @@
           <t>DE COSTER Gabriel</t>
         </is>
       </c>
-      <c r="U197" t="inlineStr">
+      <c r="X197" t="inlineStr">
         <is>
           <t>68818</t>
         </is>
@@ -11813,7 +11843,7 @@
           <t>CHAPPELL Etienne</t>
         </is>
       </c>
-      <c r="U198" t="inlineStr">
+      <c r="X198" t="inlineStr">
         <is>
           <t>75833</t>
         </is>
@@ -11871,7 +11901,7 @@
           <t>MCCREERY Alistair</t>
         </is>
       </c>
-      <c r="U199" t="inlineStr">
+      <c r="X199" t="inlineStr">
         <is>
           <t>60125</t>
         </is>
@@ -11929,7 +11959,7 @@
           <t>STANOVSKY Samuel</t>
         </is>
       </c>
-      <c r="U200" t="inlineStr">
+      <c r="X200" t="inlineStr">
         <is>
           <t>84121</t>
         </is>
@@ -11987,7 +12017,7 @@
           <t>HENDRICK Noel</t>
         </is>
       </c>
-      <c r="U201" t="inlineStr">
+      <c r="X201" t="inlineStr">
         <is>
           <t>43003</t>
         </is>
@@ -12045,7 +12075,7 @@
           <t>ALVARENGA Frederico</t>
         </is>
       </c>
-      <c r="U202" t="inlineStr">
+      <c r="X202" t="inlineStr">
         <is>
           <t>71976</t>
         </is>
@@ -12103,7 +12133,7 @@
           <t>TEAGUE Eoin</t>
         </is>
       </c>
-      <c r="U203" t="inlineStr">
+      <c r="X203" t="inlineStr">
         <is>
           <t>37913</t>
         </is>
@@ -12161,7 +12191,7 @@
           <t>WESTFALL Tyler</t>
         </is>
       </c>
-      <c r="U204" t="inlineStr">
+      <c r="X204" t="inlineStr">
         <is>
           <t>51919</t>
         </is>
@@ -12219,7 +12249,7 @@
           <t>KARLSSON Max</t>
         </is>
       </c>
-      <c r="U205" t="inlineStr">
+      <c r="X205" t="inlineStr">
         <is>
           <t>35111</t>
         </is>
@@ -12277,7 +12307,7 @@
           <t>LEE EDWARDS Ciaran</t>
         </is>
       </c>
-      <c r="U206" t="inlineStr">
+      <c r="X206" t="inlineStr">
         <is>
           <t>35614</t>
         </is>
@@ -12335,7 +12365,7 @@
           <t>THOMPSON Angus</t>
         </is>
       </c>
-      <c r="U207" t="inlineStr">
+      <c r="X207" t="inlineStr">
         <is>
           <t>44814</t>
         </is>
@@ -12393,7 +12423,7 @@
           <t>WAHLEN Fredrik</t>
         </is>
       </c>
-      <c r="U208" t="inlineStr">
+      <c r="X208" t="inlineStr">
         <is>
           <t>35102</t>
         </is>
@@ -12451,7 +12481,7 @@
           <t>POTOCNY Marcel</t>
         </is>
       </c>
-      <c r="U209" t="inlineStr">
+      <c r="X209" t="inlineStr">
         <is>
           <t>35235</t>
         </is>
@@ -12509,7 +12539,7 @@
           <t>QUAN Xin</t>
         </is>
       </c>
-      <c r="U210" t="inlineStr">
+      <c r="X210" t="inlineStr">
         <is>
           <t>62343</t>
         </is>
@@ -12567,7 +12597,7 @@
           <t>SILVA Ivan</t>
         </is>
       </c>
-      <c r="U211" t="inlineStr">
+      <c r="X211" t="inlineStr">
         <is>
           <t>35482</t>
         </is>
@@ -12625,7 +12655,7 @@
           <t>POPE Benjamin</t>
         </is>
       </c>
-      <c r="U212" t="inlineStr">
+      <c r="X212" t="inlineStr">
         <is>
           <t>51753</t>
         </is>
@@ -12683,7 +12713,7 @@
           <t>DESNOS Mathieu</t>
         </is>
       </c>
-      <c r="U213" t="inlineStr">
+      <c r="X213" t="inlineStr">
         <is>
           <t>93791</t>
         </is>
@@ -12741,7 +12771,7 @@
           <t>DELASSUS Anatole</t>
         </is>
       </c>
-      <c r="U214" t="inlineStr">
+      <c r="X214" t="inlineStr">
         <is>
           <t>84109</t>
         </is>
@@ -12799,7 +12829,7 @@
           <t>BEDA Marcello</t>
         </is>
       </c>
-      <c r="U215" t="inlineStr">
+      <c r="X215" t="inlineStr">
         <is>
           <t>39899</t>
         </is>
@@ -12857,7 +12887,7 @@
           <t>MUNSCH Manuel</t>
         </is>
       </c>
-      <c r="U216" t="inlineStr">
+      <c r="X216" t="inlineStr">
         <is>
           <t>35631</t>
         </is>
@@ -12915,7 +12945,7 @@
           <t>MAJERCZAK Krzysztof</t>
         </is>
       </c>
-      <c r="U217" t="inlineStr">
+      <c r="X217" t="inlineStr">
         <is>
           <t>53647</t>
         </is>
@@ -12973,7 +13003,7 @@
           <t>BURGI Quentin</t>
         </is>
       </c>
-      <c r="U218" t="inlineStr">
+      <c r="X218" t="inlineStr">
         <is>
           <t>41590</t>
         </is>
@@ -13031,7 +13061,7 @@
           <t>GILBERT Callum</t>
         </is>
       </c>
-      <c r="U219" t="inlineStr">
+      <c r="X219" t="inlineStr">
         <is>
           <t>42090</t>
         </is>
@@ -13089,7 +13119,7 @@
           <t>LEITNER Mario</t>
         </is>
       </c>
-      <c r="U220" t="inlineStr">
+      <c r="X220" t="inlineStr">
         <is>
           <t>35546</t>
         </is>
@@ -13147,7 +13177,7 @@
           <t>MAXEINER Tim</t>
         </is>
       </c>
-      <c r="U221" t="inlineStr">
+      <c r="X221" t="inlineStr">
         <is>
           <t>35117</t>
         </is>
@@ -13205,7 +13235,7 @@
           <t>TESTEN Niko</t>
         </is>
       </c>
-      <c r="U222" t="inlineStr">
+      <c r="X222" t="inlineStr">
         <is>
           <t>39980</t>
         </is>
@@ -13263,7 +13293,7 @@
           <t>SRABOTNIK Martin</t>
         </is>
       </c>
-      <c r="U223" t="inlineStr">
+      <c r="X223" t="inlineStr">
         <is>
           <t>39080</t>
         </is>
@@ -13321,7 +13351,7 @@
           <t>HERNANZ Samuel</t>
         </is>
       </c>
-      <c r="U224" t="inlineStr">
+      <c r="X224" t="inlineStr">
         <is>
           <t>35786</t>
         </is>
@@ -13379,7 +13409,7 @@
           <t>OHRSTROM Isak</t>
         </is>
       </c>
-      <c r="U225" t="inlineStr">
+      <c r="X225" t="inlineStr">
         <is>
           <t>35101</t>
         </is>
@@ -13437,7 +13467,7 @@
           <t>HRADILEK Vavrinec</t>
         </is>
       </c>
-      <c r="U226" t="inlineStr">
+      <c r="X226" t="inlineStr">
         <is>
           <t>35031</t>
         </is>
@@ -13495,7 +13525,7 @@
           <t>SCHWEIKERT Fabian</t>
         </is>
       </c>
-      <c r="U227" t="inlineStr">
+      <c r="X227" t="inlineStr">
         <is>
           <t>38412</t>
         </is>
@@ -13553,7 +13583,7 @@
           <t>IVALDI Zeno</t>
         </is>
       </c>
-      <c r="U228" t="inlineStr">
+      <c r="X228" t="inlineStr">
         <is>
           <t>35480</t>
         </is>
@@ -13611,7 +13641,7 @@
           <t>OSCHMAUTZ Felix</t>
         </is>
       </c>
-      <c r="U229" t="inlineStr">
+      <c r="X229" t="inlineStr">
         <is>
           <t>51856</t>
         </is>
@@ -13669,7 +13699,7 @@
           <t>MALEK Andrej</t>
         </is>
       </c>
-      <c r="U230" t="inlineStr">
+      <c r="X230" t="inlineStr">
         <is>
           <t>39246</t>
         </is>
@@ -13727,7 +13757,7 @@
           <t>HALCIN Martin</t>
         </is>
       </c>
-      <c r="U231" t="inlineStr">
+      <c r="X231" t="inlineStr">
         <is>
           <t>35355</t>
         </is>
@@ -13785,7 +13815,7 @@
           <t>WERRO Lukas</t>
         </is>
       </c>
-      <c r="U232" t="inlineStr">
+      <c r="X232" t="inlineStr">
         <is>
           <t>35347</t>
         </is>
@@ -13843,7 +13873,7 @@
           <t>LAUNAY Antoine</t>
         </is>
       </c>
-      <c r="U233" t="inlineStr">
+      <c r="X233" t="inlineStr">
         <is>
           <t>68776</t>
         </is>
@@ -13901,7 +13931,7 @@
           <t>LLORENTE David</t>
         </is>
       </c>
-      <c r="U234" t="inlineStr">
+      <c r="X234" t="inlineStr">
         <is>
           <t>51850</t>
         </is>
@@ -13959,7 +13989,7 @@
           <t>CRESPO Joan</t>
         </is>
       </c>
-      <c r="U235" t="inlineStr">
+      <c r="X235" t="inlineStr">
         <is>
           <t>35749</t>
         </is>
@@ -14017,7 +14047,7 @@
           <t>PASIUT Michal</t>
         </is>
       </c>
-      <c r="U236" t="inlineStr">
+      <c r="X236" t="inlineStr">
         <is>
           <t>35095</t>
         </is>
@@ -14075,7 +14105,7 @@
           <t>DOUGOUD Martin</t>
         </is>
       </c>
-      <c r="U237" t="inlineStr">
+      <c r="X237" t="inlineStr">
         <is>
           <t>35426</t>
         </is>
@@ -14133,7 +14163,7 @@
           <t>GRIGAR Jakub</t>
         </is>
       </c>
-      <c r="U238" t="inlineStr">
+      <c r="X238" t="inlineStr">
         <is>
           <t>37284</t>
         </is>
@@ -14191,7 +14221,7 @@
           <t>SMOLEN Michal</t>
         </is>
       </c>
-      <c r="U239" t="inlineStr">
+      <c r="X239" t="inlineStr">
         <is>
           <t>36397</t>
         </is>
@@ -14249,7 +14279,7 @@
           <t>POPIELA Dariusz</t>
         </is>
       </c>
-      <c r="U240" t="inlineStr">
+      <c r="X240" t="inlineStr">
         <is>
           <t>35096</t>
         </is>
@@ -14307,7 +14337,7 @@
           <t>DE GENNARO Giovanni</t>
         </is>
       </c>
-      <c r="U241" t="inlineStr">
+      <c r="X241" t="inlineStr">
         <is>
           <t>35244</t>
         </is>
@@ -14365,7 +14395,7 @@
           <t>DELFOUR Lucien</t>
         </is>
       </c>
-      <c r="U242" t="inlineStr">
+      <c r="X242" t="inlineStr">
         <is>
           <t>36537</t>
         </is>
@@ -14423,7 +14453,7 @@
           <t>AIGNER Hannes</t>
         </is>
       </c>
-      <c r="U243" t="inlineStr">
+      <c r="X243" t="inlineStr">
         <is>
           <t>35115</t>
         </is>
@@ -14481,7 +14511,7 @@
           <t>PRINDIS Vit</t>
         </is>
       </c>
-      <c r="U244" t="inlineStr">
+      <c r="X244" t="inlineStr">
         <is>
           <t>35065</t>
         </is>
@@ -14539,7 +14569,7 @@
           <t>NEVEU Boris</t>
         </is>
       </c>
-      <c r="U245" t="inlineStr">
+      <c r="X245" t="inlineStr">
         <is>
           <t>35396</t>
         </is>
@@ -14597,7 +14627,7 @@
           <t>PRSKAVEC Jiri</t>
         </is>
       </c>
-      <c r="U246" t="inlineStr">
+      <c r="X246" t="inlineStr">
         <is>
           <t>35033</t>
         </is>
@@ -14655,7 +14685,7 @@
           <t>KAUZER Peter</t>
         </is>
       </c>
-      <c r="U247" t="inlineStr">
+      <c r="X247" t="inlineStr">
         <is>
           <t>35589</t>
         </is>
@@ -14713,7 +14743,7 @@
           <t>ZWOLINSKA Klaudia</t>
         </is>
       </c>
-      <c r="U248" t="inlineStr">
+      <c r="X248" t="inlineStr">
         <is>
           <t>42027</t>
         </is>
@@ -14771,7 +14801,7 @@
           <t>YU Cuishan</t>
         </is>
       </c>
-      <c r="U249" t="inlineStr">
+      <c r="X249" t="inlineStr">
         <is>
           <t>75380</t>
         </is>
@@ -14829,7 +14859,7 @@
           <t>LAMEIRO Ainhoa</t>
         </is>
       </c>
-      <c r="U250" t="inlineStr">
+      <c r="X250" t="inlineStr">
         <is>
           <t>69042</t>
         </is>
@@ -14887,7 +14917,7 @@
           <t>TENG Qianqian</t>
         </is>
       </c>
-      <c r="U251" t="inlineStr">
+      <c r="X251" t="inlineStr">
         <is>
           <t>94209</t>
         </is>
@@ -14945,7 +14975,7 @@
           <t>MARX Alena</t>
         </is>
       </c>
-      <c r="U252" t="inlineStr">
+      <c r="X252" t="inlineStr">
         <is>
           <t>68844</t>
         </is>
@@ -15003,7 +15033,7 @@
           <t>SPICER Phoebe</t>
         </is>
       </c>
-      <c r="U253" t="inlineStr">
+      <c r="X253" t="inlineStr">
         <is>
           <t>75827</t>
         </is>
@@ -15061,7 +15091,7 @@
           <t>NOVAK Lea</t>
         </is>
       </c>
-      <c r="U254" t="inlineStr">
+      <c r="X254" t="inlineStr">
         <is>
           <t>60323</t>
         </is>
@@ -15119,7 +15149,7 @@
           <t>YAGI Airi</t>
         </is>
       </c>
-      <c r="U255" t="inlineStr">
+      <c r="X255" t="inlineStr">
         <is>
           <t>37756</t>
         </is>
@@ -15177,7 +15207,7 @@
           <t>STACH Aleksandra</t>
         </is>
       </c>
-      <c r="U256" t="inlineStr">
+      <c r="X256" t="inlineStr">
         <is>
           <t>61261</t>
         </is>
@@ -15235,7 +15265,7 @@
           <t>LUKNAROVA Emanuela</t>
         </is>
       </c>
-      <c r="U257" t="inlineStr">
+      <c r="X257" t="inlineStr">
         <is>
           <t>76973</t>
         </is>
@@ -15293,7 +15323,7 @@
           <t>HAVLICKOVA Katerina</t>
         </is>
       </c>
-      <c r="U258" t="inlineStr">
+      <c r="X258" t="inlineStr">
         <is>
           <t>35048</t>
         </is>
@@ -15351,7 +15381,7 @@
           <t>FORROW Bethan</t>
         </is>
       </c>
-      <c r="U259" t="inlineStr">
+      <c r="X259" t="inlineStr">
         <is>
           <t>69065</t>
         </is>
@@ -15409,7 +15439,7 @@
           <t>DELASSUS Marjorie</t>
         </is>
       </c>
-      <c r="U260" t="inlineStr">
+      <c r="X260" t="inlineStr">
         <is>
           <t>71964</t>
         </is>
@@ -15467,7 +15497,7 @@
           <t>KOZOROG Alja</t>
         </is>
       </c>
-      <c r="U261" t="inlineStr">
+      <c r="X261" t="inlineStr">
         <is>
           <t>39986</t>
         </is>
@@ -15525,7 +15555,7 @@
           <t>SKACHOVA Monika</t>
         </is>
       </c>
-      <c r="U262" t="inlineStr">
+      <c r="X262" t="inlineStr">
         <is>
           <t>53078</t>
         </is>
@@ -15583,7 +15613,7 @@
           <t>STANOVSKA Sona</t>
         </is>
       </c>
-      <c r="U263" t="inlineStr">
+      <c r="X263" t="inlineStr">
         <is>
           <t>51647</t>
         </is>
@@ -15641,7 +15671,7 @@
           <t>DORIA VILARRUBLA Monica</t>
         </is>
       </c>
-      <c r="U264" t="inlineStr">
+      <c r="X264" t="inlineStr">
         <is>
           <t>53051</t>
         </is>
@@ -15699,7 +15729,7 @@
           <t>WOLFFHARDT Viktoria</t>
         </is>
       </c>
-      <c r="U265" t="inlineStr">
+      <c r="X265" t="inlineStr">
         <is>
           <t>35303</t>
         </is>
@@ -15757,7 +15787,7 @@
           <t>CHEN Tianlu</t>
         </is>
       </c>
-      <c r="U266" t="inlineStr">
+      <c r="X266" t="inlineStr">
         <is>
           <t>84748</t>
         </is>
@@ -15815,7 +15845,7 @@
           <t>CELMINS Ritvars</t>
         </is>
       </c>
-      <c r="U267" t="inlineStr">
+      <c r="X267" t="inlineStr">
         <is>
           <t>35182</t>
         </is>
@@ -15873,7 +15903,7 @@
           <t>KOJIMA Daichi</t>
         </is>
       </c>
-      <c r="U268" t="inlineStr">
+      <c r="X268" t="inlineStr">
         <is>
           <t>42255</t>
         </is>
@@ -15931,7 +15961,7 @@
           <t>SWETNAM Huw</t>
         </is>
       </c>
-      <c r="U269" t="inlineStr">
+      <c r="X269" t="inlineStr">
         <is>
           <t>35652</t>
         </is>
@@ -15989,7 +16019,7 @@
           <t>MUTO Yusuke</t>
         </is>
       </c>
-      <c r="U270" t="inlineStr">
+      <c r="X270" t="inlineStr">
         <is>
           <t>71820</t>
         </is>
@@ -16047,7 +16077,7 @@
           <t>TANAKA Yuuki</t>
         </is>
       </c>
-      <c r="U271" t="inlineStr">
+      <c r="X271" t="inlineStr">
         <is>
           <t>75422</t>
         </is>
@@ -16105,7 +16135,7 @@
           <t>DE COSTER Gabriel</t>
         </is>
       </c>
-      <c r="U272" t="inlineStr">
+      <c r="X272" t="inlineStr">
         <is>
           <t>68818</t>
         </is>
@@ -16163,7 +16193,7 @@
           <t>CHAPPELL Etienne</t>
         </is>
       </c>
-      <c r="U273" t="inlineStr">
+      <c r="X273" t="inlineStr">
         <is>
           <t>75833</t>
         </is>
@@ -16221,7 +16251,7 @@
           <t>MCCREERY Alistair</t>
         </is>
       </c>
-      <c r="U274" t="inlineStr">
+      <c r="X274" t="inlineStr">
         <is>
           <t>60125</t>
         </is>
@@ -16279,7 +16309,7 @@
           <t>STANOVSKY Samuel</t>
         </is>
       </c>
-      <c r="U275" t="inlineStr">
+      <c r="X275" t="inlineStr">
         <is>
           <t>84121</t>
         </is>
@@ -16337,7 +16367,7 @@
           <t>HENDRICK Noel</t>
         </is>
       </c>
-      <c r="U276" t="inlineStr">
+      <c r="X276" t="inlineStr">
         <is>
           <t>43003</t>
         </is>
@@ -16395,7 +16425,7 @@
           <t>ALVARENGA Frederico</t>
         </is>
       </c>
-      <c r="U277" t="inlineStr">
+      <c r="X277" t="inlineStr">
         <is>
           <t>71976</t>
         </is>
@@ -16453,7 +16483,7 @@
           <t>TEAGUE Eoin</t>
         </is>
       </c>
-      <c r="U278" t="inlineStr">
+      <c r="X278" t="inlineStr">
         <is>
           <t>37913</t>
         </is>
@@ -16511,7 +16541,7 @@
           <t>WESTFALL Tyler</t>
         </is>
       </c>
-      <c r="U279" t="inlineStr">
+      <c r="X279" t="inlineStr">
         <is>
           <t>51919</t>
         </is>
@@ -16569,7 +16599,7 @@
           <t>LEE EDWARDS Ciaran</t>
         </is>
       </c>
-      <c r="U280" t="inlineStr">
+      <c r="X280" t="inlineStr">
         <is>
           <t>35614</t>
         </is>
@@ -16627,7 +16657,7 @@
           <t>POTOCNY Marcel</t>
         </is>
       </c>
-      <c r="U281" t="inlineStr">
+      <c r="X281" t="inlineStr">
         <is>
           <t>35235</t>
         </is>
@@ -16685,7 +16715,7 @@
           <t>SILVA Ivan</t>
         </is>
       </c>
-      <c r="U282" t="inlineStr">
+      <c r="X282" t="inlineStr">
         <is>
           <t>35482</t>
         </is>
@@ -16743,7 +16773,7 @@
           <t>DESNOS Mathieu</t>
         </is>
       </c>
-      <c r="U283" t="inlineStr">
+      <c r="X283" t="inlineStr">
         <is>
           <t>93791</t>
         </is>
@@ -16801,7 +16831,7 @@
           <t>MUNSCH Manuel</t>
         </is>
       </c>
-      <c r="U284" t="inlineStr">
+      <c r="X284" t="inlineStr">
         <is>
           <t>35631</t>
         </is>
@@ -16859,7 +16889,7 @@
           <t>LEITNER Mario</t>
         </is>
       </c>
-      <c r="U285" t="inlineStr">
+      <c r="X285" t="inlineStr">
         <is>
           <t>35546</t>
         </is>
@@ -16917,7 +16947,7 @@
           <t>TESTEN Niko</t>
         </is>
       </c>
-      <c r="U286" t="inlineStr">
+      <c r="X286" t="inlineStr">
         <is>
           <t>39980</t>
         </is>
@@ -16975,7 +17005,7 @@
           <t>SCHWEIKERT Fabian</t>
         </is>
       </c>
-      <c r="U287" t="inlineStr">
+      <c r="X287" t="inlineStr">
         <is>
           <t>38412</t>
         </is>
@@ -17033,7 +17063,7 @@
           <t>MALEK Andrej</t>
         </is>
       </c>
-      <c r="U288" t="inlineStr">
+      <c r="X288" t="inlineStr">
         <is>
           <t>39246</t>
         </is>
@@ -17091,7 +17121,7 @@
           <t>LLORENTE David</t>
         </is>
       </c>
-      <c r="U289" t="inlineStr">
+      <c r="X289" t="inlineStr">
         <is>
           <t>51850</t>
         </is>
@@ -17149,7 +17179,7 @@
           <t>PASIUT Michal</t>
         </is>
       </c>
-      <c r="U290" t="inlineStr">
+      <c r="X290" t="inlineStr">
         <is>
           <t>35095</t>
         </is>
@@ -17207,7 +17237,7 @@
           <t>GRIGAR Jakub</t>
         </is>
       </c>
-      <c r="U291" t="inlineStr">
+      <c r="X291" t="inlineStr">
         <is>
           <t>37284</t>
         </is>
@@ -17265,7 +17295,7 @@
           <t>NEVEU Boris</t>
         </is>
       </c>
-      <c r="U292" t="inlineStr">
+      <c r="X292" t="inlineStr">
         <is>
           <t>35396</t>
         </is>
@@ -17909,7 +17939,7 @@
           <t>CONEY William</t>
         </is>
       </c>
-      <c r="U305" t="inlineStr">
+      <c r="X305" t="inlineStr">
         <is>
           <t>53138</t>
         </is>
@@ -18020,7 +18050,7 @@
           <t>ROISIN Lucas</t>
         </is>
       </c>
-      <c r="U307" t="inlineStr">
+      <c r="X307" t="inlineStr">
         <is>
           <t>55580</t>
         </is>
@@ -18078,7 +18108,7 @@
           <t>COCHRANE Jake</t>
         </is>
       </c>
-      <c r="U308" t="inlineStr">
+      <c r="X308" t="inlineStr">
         <is>
           <t>60124</t>
         </is>
@@ -18136,7 +18166,7 @@
           <t>CRAWFORD Brodie</t>
         </is>
       </c>
-      <c r="U309" t="inlineStr">
+      <c r="X309" t="inlineStr">
         <is>
           <t>38436</t>
         </is>
@@ -18194,7 +18224,7 @@
           <t>KOECHLIN Thomas</t>
         </is>
       </c>
-      <c r="U310" t="inlineStr">
+      <c r="X310" t="inlineStr">
         <is>
           <t>35419</t>
         </is>
@@ -18252,7 +18282,7 @@
           <t>CARTER Tristan</t>
         </is>
       </c>
-      <c r="U311" t="inlineStr">
+      <c r="X311" t="inlineStr">
         <is>
           <t>51890</t>
         </is>
@@ -18310,7 +18340,7 @@
           <t>GESTIN Nicolas</t>
         </is>
       </c>
-      <c r="U312" t="inlineStr">
+      <c r="X312" t="inlineStr">
         <is>
           <t>71961</t>
         </is>
@@ -18368,7 +18398,7 @@
           <t>HEDWIG Grzegorz</t>
         </is>
       </c>
-      <c r="U313" t="inlineStr">
+      <c r="X313" t="inlineStr">
         <is>
           <t>35465</t>
         </is>
@@ -18426,7 +18456,7 @@
           <t>CARVALHO Jose</t>
         </is>
       </c>
-      <c r="U314" t="inlineStr">
+      <c r="X314" t="inlineStr">
         <is>
           <t>35486</t>
         </is>
@@ -18484,7 +18514,7 @@
           <t>RAK Tomas</t>
         </is>
       </c>
-      <c r="U315" t="inlineStr">
+      <c r="X315" t="inlineStr">
         <is>
           <t>35056</t>
         </is>
@@ -18542,7 +18572,7 @@
           <t>COLAZINGARI Roberto</t>
         </is>
       </c>
-      <c r="U316" t="inlineStr">
+      <c r="X316" t="inlineStr">
         <is>
           <t>35223</t>
         </is>
@@ -18600,7 +18630,7 @@
           <t>ELOSEGI Ander</t>
         </is>
       </c>
-      <c r="U317" t="inlineStr">
+      <c r="X317" t="inlineStr">
         <is>
           <t>35785</t>
         </is>
@@ -18658,7 +18688,7 @@
           <t>HEGER Vojtech</t>
         </is>
       </c>
-      <c r="U318" t="inlineStr">
+      <c r="X318" t="inlineStr">
         <is>
           <t>68872</t>
         </is>
@@ -18716,7 +18746,7 @@
           <t>ABBOTT Thomas</t>
         </is>
       </c>
-      <c r="U319" t="inlineStr">
+      <c r="X319" t="inlineStr">
         <is>
           <t>36514</t>
         </is>
@@ -18774,7 +18804,7 @@
           <t>BERCIC Anze</t>
         </is>
       </c>
-      <c r="U320" t="inlineStr">
+      <c r="X320" t="inlineStr">
         <is>
           <t>36253</t>
         </is>
@@ -18832,7 +18862,7 @@
           <t>IVALDI Raffaello</t>
         </is>
       </c>
-      <c r="U321" t="inlineStr">
+      <c r="X321" t="inlineStr">
         <is>
           <t>35227</t>
         </is>
@@ -18890,7 +18920,7 @@
           <t>SZTUBA Kacper</t>
         </is>
       </c>
-      <c r="U322" t="inlineStr">
+      <c r="X322" t="inlineStr">
         <is>
           <t>53636</t>
         </is>
@@ -18948,7 +18978,7 @@
           <t>ANTON Franz</t>
         </is>
       </c>
-      <c r="U323" t="inlineStr">
+      <c r="X323" t="inlineStr">
         <is>
           <t>35137</t>
         </is>
@@ -19006,7 +19036,7 @@
           <t>LOKKEN Zachary</t>
         </is>
       </c>
-      <c r="U324" t="inlineStr">
+      <c r="X324" t="inlineStr">
         <is>
           <t>35069</t>
         </is>
@@ -19064,7 +19094,7 @@
           <t>CIPRESSI Stefano</t>
         </is>
       </c>
-      <c r="U325" t="inlineStr">
+      <c r="X325" t="inlineStr">
         <is>
           <t>35495</t>
         </is>
@@ -19122,7 +19152,7 @@
           <t>GARGAUD CHANUT Denis</t>
         </is>
       </c>
-      <c r="U326" t="inlineStr">
+      <c r="X326" t="inlineStr">
         <is>
           <t>35177</t>
         </is>
@@ -19180,7 +19210,7 @@
           <t>BOZIC Luka</t>
         </is>
       </c>
-      <c r="U327" t="inlineStr">
+      <c r="X327" t="inlineStr">
         <is>
           <t>36269</t>
         </is>
@@ -19238,7 +19268,7 @@
           <t>MARTIKAN Michal</t>
         </is>
       </c>
-      <c r="U328" t="inlineStr">
+      <c r="X328" t="inlineStr">
         <is>
           <t>35365</t>
         </is>
@@ -19296,7 +19326,7 @@
           <t>BENUS Matej</t>
         </is>
       </c>
-      <c r="U329" t="inlineStr">
+      <c r="X329" t="inlineStr">
         <is>
           <t>35353</t>
         </is>
@@ -19354,7 +19384,7 @@
           <t>SAVSEK Benjamin</t>
         </is>
       </c>
-      <c r="U330" t="inlineStr">
+      <c r="X330" t="inlineStr">
         <is>
           <t>36218</t>
         </is>
@@ -19412,7 +19442,7 @@
           <t>ROHAN Lukas</t>
         </is>
       </c>
-      <c r="U331" t="inlineStr">
+      <c r="X331" t="inlineStr">
         <is>
           <t>36114</t>
         </is>
@@ -19470,7 +19500,7 @@
           <t>TRAVE Miquel</t>
         </is>
       </c>
-      <c r="U332" t="inlineStr">
+      <c r="X332" t="inlineStr">
         <is>
           <t>68998</t>
         </is>
@@ -19528,7 +19558,7 @@
           <t>SLAFKOVSKY Alexander</t>
         </is>
       </c>
-      <c r="U333" t="inlineStr">
+      <c r="X333" t="inlineStr">
         <is>
           <t>35129</t>
         </is>
@@ -19586,7 +19616,7 @@
           <t>TASIADIS Sideris</t>
         </is>
       </c>
-      <c r="U334" t="inlineStr">
+      <c r="X334" t="inlineStr">
         <is>
           <t>35135</t>
         </is>
@@ -19644,7 +19674,7 @@
           <t>DORIA VILARRUBLA Monica</t>
         </is>
       </c>
-      <c r="U335" t="inlineStr">
+      <c r="X335" t="inlineStr">
         <is>
           <t>53051</t>
         </is>
@@ -19702,7 +19732,7 @@
           <t>WEGMAN Martina</t>
         </is>
       </c>
-      <c r="U336" t="inlineStr">
+      <c r="X336" t="inlineStr">
         <is>
           <t>35345</t>
         </is>
@@ -19760,7 +19790,7 @@
           <t>SETCHELL Nikita</t>
         </is>
       </c>
-      <c r="U337" t="inlineStr">
+      <c r="X337" t="inlineStr">
         <is>
           <t>86250</t>
         </is>
@@ -19818,7 +19848,7 @@
           <t>HOCEVAR Eva Alina</t>
         </is>
       </c>
-      <c r="U338" t="inlineStr">
+      <c r="X338" t="inlineStr">
         <is>
           <t>75533</t>
         </is>
@@ -19876,7 +19906,7 @@
           <t>TEUNISSEN Lena</t>
         </is>
       </c>
-      <c r="U339" t="inlineStr">
+      <c r="X339" t="inlineStr">
         <is>
           <t>35344</t>
         </is>
@@ -19934,7 +19964,7 @@
           <t>VOJTOVA Veronika</t>
         </is>
       </c>
-      <c r="U340" t="inlineStr">
+      <c r="X340" t="inlineStr">
         <is>
           <t>35945</t>
         </is>
@@ -19992,7 +20022,7 @@
           <t>WERATSCHNIG Nina</t>
         </is>
       </c>
-      <c r="U341" t="inlineStr">
+      <c r="X341" t="inlineStr">
         <is>
           <t>41614</t>
         </is>
@@ -20050,7 +20080,7 @@
           <t>HILGERTOVA Amalie</t>
         </is>
       </c>
-      <c r="U342" t="inlineStr">
+      <c r="X342" t="inlineStr">
         <is>
           <t>36113</t>
         </is>
@@ -20108,7 +20138,7 @@
           <t>DUKATOVA Jana</t>
         </is>
       </c>
-      <c r="U343" t="inlineStr">
+      <c r="X343" t="inlineStr">
         <is>
           <t>35354</t>
         </is>
@@ -20166,7 +20196,7 @@
           <t>MINTALOVA Eliska</t>
         </is>
       </c>
-      <c r="U344" t="inlineStr">
+      <c r="X344" t="inlineStr">
         <is>
           <t>56169</t>
         </is>
@@ -20224,7 +20254,7 @@
           <t>LEENDERS Claudia</t>
         </is>
       </c>
-      <c r="U345" t="inlineStr">
+      <c r="X345" t="inlineStr">
         <is>
           <t>35331</t>
         </is>
@@ -20282,7 +20312,7 @@
           <t>LEIBFARTH Evy</t>
         </is>
       </c>
-      <c r="U346" t="inlineStr">
+      <c r="X346" t="inlineStr">
         <is>
           <t>83538</t>
         </is>
@@ -20340,7 +20370,7 @@
           <t>KALISKA Elena</t>
         </is>
       </c>
-      <c r="U347" t="inlineStr">
+      <c r="X347" t="inlineStr">
         <is>
           <t>35366</t>
         </is>
@@ -20398,7 +20428,7 @@
           <t>WOLFFHARDT Viktoria</t>
         </is>
       </c>
-      <c r="U348" t="inlineStr">
+      <c r="X348" t="inlineStr">
         <is>
           <t>35303</t>
         </is>
@@ -20456,7 +20486,7 @@
           <t>ZWOLINSKA Klaudia</t>
         </is>
       </c>
-      <c r="U349" t="inlineStr">
+      <c r="X349" t="inlineStr">
         <is>
           <t>42027</t>
         </is>
@@ -20514,7 +20544,7 @@
           <t>KUHNLE Corinna</t>
         </is>
       </c>
-      <c r="U350" t="inlineStr">
+      <c r="X350" t="inlineStr">
         <is>
           <t>35282</t>
         </is>
@@ -20572,7 +20602,7 @@
           <t>LAFONT Marie-Zelia</t>
         </is>
       </c>
-      <c r="U351" t="inlineStr">
+      <c r="X351" t="inlineStr">
         <is>
           <t>35374</t>
         </is>
@@ -20630,7 +20660,7 @@
           <t>APEL Elena</t>
         </is>
       </c>
-      <c r="U352" t="inlineStr">
+      <c r="X352" t="inlineStr">
         <is>
           <t>51837</t>
         </is>
@@ -20688,7 +20718,7 @@
           <t>HAMER-EVANS Megan</t>
         </is>
       </c>
-      <c r="U353" t="inlineStr">
+      <c r="X353" t="inlineStr">
         <is>
           <t>55138</t>
         </is>
@@ -20746,7 +20776,7 @@
           <t>HORN Stefanie</t>
         </is>
       </c>
-      <c r="U354" t="inlineStr">
+      <c r="X354" t="inlineStr">
         <is>
           <t>38417</t>
         </is>
@@ -20804,7 +20834,7 @@
           <t>KUDEJOVA Katerina</t>
         </is>
       </c>
-      <c r="U355" t="inlineStr">
+      <c r="X355" t="inlineStr">
         <is>
           <t>35034</t>
         </is>
@@ -20862,7 +20892,7 @@
           <t>TERCELJ Eva</t>
         </is>
       </c>
-      <c r="U356" t="inlineStr">
+      <c r="X356" t="inlineStr">
         <is>
           <t>36263</t>
         </is>
@@ -20920,7 +20950,7 @@
           <t>SCHORNBERG Jasmin</t>
         </is>
       </c>
-      <c r="U357" t="inlineStr">
+      <c r="X357" t="inlineStr">
         <is>
           <t>35206</t>
         </is>
@@ -20978,7 +21008,7 @@
           <t>CHOURRAUT Maialen</t>
         </is>
       </c>
-      <c r="U358" t="inlineStr">
+      <c r="X358" t="inlineStr">
         <is>
           <t>35787</t>
         </is>
@@ -21036,7 +21066,7 @@
           <t>PRIGENT Camille</t>
         </is>
       </c>
-      <c r="U359" t="inlineStr">
+      <c r="X359" t="inlineStr">
         <is>
           <t>41566</t>
         </is>
@@ -21094,7 +21124,7 @@
           <t>SATILA Ana</t>
         </is>
       </c>
-      <c r="U360" t="inlineStr">
+      <c r="X360" t="inlineStr">
         <is>
           <t>35327</t>
         </is>
@@ -21152,7 +21182,7 @@
           <t>BAUDU Lucie</t>
         </is>
       </c>
-      <c r="U361" t="inlineStr">
+      <c r="X361" t="inlineStr">
         <is>
           <t>35669</t>
         </is>
@@ -21210,7 +21240,7 @@
           <t>PACIERPNIK Natalia</t>
         </is>
       </c>
-      <c r="U362" t="inlineStr">
+      <c r="X362" t="inlineStr">
         <is>
           <t>35077</t>
         </is>
@@ -21268,7 +21298,7 @@
           <t>FOX Jessica</t>
         </is>
       </c>
-      <c r="U363" t="inlineStr">
+      <c r="X363" t="inlineStr">
         <is>
           <t>36526</t>
         </is>
@@ -21326,7 +21356,7 @@
           <t>FUNK Ricarda</t>
         </is>
       </c>
-      <c r="U364" t="inlineStr">
+      <c r="X364" t="inlineStr">
         <is>
           <t>35122</t>
         </is>
@@ -21394,7 +21424,7 @@
           <t>BENUS Matej</t>
         </is>
       </c>
-      <c r="U365" t="inlineStr">
+      <c r="X365" t="inlineStr">
         <is>
           <t>35353</t>
         </is>
@@ -21462,7 +21492,7 @@
           <t>CIPRESSI Stefano</t>
         </is>
       </c>
-      <c r="U366" t="inlineStr">
+      <c r="X366" t="inlineStr">
         <is>
           <t>35495</t>
         </is>
@@ -21530,7 +21560,7 @@
           <t>IVALDI Raffaello</t>
         </is>
       </c>
-      <c r="U367" t="inlineStr">
+      <c r="X367" t="inlineStr">
         <is>
           <t>35227</t>
         </is>
@@ -21598,7 +21628,7 @@
           <t>ELOSEGI Ander</t>
         </is>
       </c>
-      <c r="U368" t="inlineStr">
+      <c r="X368" t="inlineStr">
         <is>
           <t>35785</t>
         </is>
@@ -21666,7 +21696,7 @@
           <t>BOZIC Luka</t>
         </is>
       </c>
-      <c r="U369" t="inlineStr">
+      <c r="X369" t="inlineStr">
         <is>
           <t>36269</t>
         </is>
@@ -21734,7 +21764,7 @@
           <t>ANTON Franz</t>
         </is>
       </c>
-      <c r="U370" t="inlineStr">
+      <c r="X370" t="inlineStr">
         <is>
           <t>35137</t>
         </is>
@@ -21802,7 +21832,7 @@
           <t>TASIADIS Sideris</t>
         </is>
       </c>
-      <c r="U371" t="inlineStr">
+      <c r="X371" t="inlineStr">
         <is>
           <t>35135</t>
         </is>
@@ -21870,7 +21900,7 @@
           <t>SAVSEK Benjamin</t>
         </is>
       </c>
-      <c r="U372" t="inlineStr">
+      <c r="X372" t="inlineStr">
         <is>
           <t>36218</t>
         </is>
@@ -21938,7 +21968,7 @@
           <t>MARTIKAN Michal</t>
         </is>
       </c>
-      <c r="U373" t="inlineStr">
+      <c r="X373" t="inlineStr">
         <is>
           <t>35365</t>
         </is>
@@ -22006,7 +22036,7 @@
           <t>SLAFKOVSKY Alexander</t>
         </is>
       </c>
-      <c r="U374" t="inlineStr">
+      <c r="X374" t="inlineStr">
         <is>
           <t>35129</t>
         </is>
@@ -22074,7 +22104,7 @@
           <t>SATILA Ana</t>
         </is>
       </c>
-      <c r="U375" t="inlineStr">
+      <c r="X375" t="inlineStr">
         <is>
           <t>35327</t>
         </is>
@@ -22142,7 +22172,7 @@
           <t>HORN Stefanie</t>
         </is>
       </c>
-      <c r="U376" t="inlineStr">
+      <c r="X376" t="inlineStr">
         <is>
           <t>38417</t>
         </is>
@@ -22210,7 +22240,7 @@
           <t>FOX Jessica</t>
         </is>
       </c>
-      <c r="U377" t="inlineStr">
+      <c r="X377" t="inlineStr">
         <is>
           <t>36526</t>
         </is>
@@ -22278,7 +22308,7 @@
           <t>SCHORNBERG Jasmin</t>
         </is>
       </c>
-      <c r="U378" t="inlineStr">
+      <c r="X378" t="inlineStr">
         <is>
           <t>35206</t>
         </is>
@@ -22346,7 +22376,7 @@
           <t>KUHNLE Corinna</t>
         </is>
       </c>
-      <c r="U379" t="inlineStr">
+      <c r="X379" t="inlineStr">
         <is>
           <t>35282</t>
         </is>
@@ -22414,7 +22444,7 @@
           <t>PRIGENT Camille</t>
         </is>
       </c>
-      <c r="U380" t="inlineStr">
+      <c r="X380" t="inlineStr">
         <is>
           <t>41566</t>
         </is>
@@ -22482,7 +22512,7 @@
           <t>ZWOLINSKA Klaudia</t>
         </is>
       </c>
-      <c r="U381" t="inlineStr">
+      <c r="X381" t="inlineStr">
         <is>
           <t>42027</t>
         </is>
@@ -22550,7 +22580,7 @@
           <t>CHOURRAUT Maialen</t>
         </is>
       </c>
-      <c r="U382" t="inlineStr">
+      <c r="X382" t="inlineStr">
         <is>
           <t>35787</t>
         </is>
@@ -22618,7 +22648,7 @@
           <t>KUDEJOVA Katerina</t>
         </is>
       </c>
-      <c r="U383" t="inlineStr">
+      <c r="X383" t="inlineStr">
         <is>
           <t>35034</t>
         </is>
@@ -22686,7 +22716,7 @@
           <t>FUNK Ricarda</t>
         </is>
       </c>
-      <c r="U384" t="inlineStr">
+      <c r="X384" t="inlineStr">
         <is>
           <t>35122</t>
         </is>
@@ -22956,7 +22986,7 @@
           <t>HAVLICKOVA Katerina</t>
         </is>
       </c>
-      <c r="U389" t="inlineStr">
+      <c r="X389" t="inlineStr">
         <is>
           <t>35048</t>
         </is>
@@ -23014,7 +23044,7 @@
           <t>TENG Qianqian</t>
         </is>
       </c>
-      <c r="U390" t="inlineStr">
+      <c r="X390" t="inlineStr">
         <is>
           <t>94209</t>
         </is>
@@ -23072,7 +23102,7 @@
           <t>LAMEIRO Ainhoa</t>
         </is>
       </c>
-      <c r="U391" t="inlineStr">
+      <c r="X391" t="inlineStr">
         <is>
           <t>69042</t>
         </is>
@@ -23130,7 +23160,7 @@
           <t>LUKNAROVA Emanuela</t>
         </is>
       </c>
-      <c r="U392" t="inlineStr">
+      <c r="X392" t="inlineStr">
         <is>
           <t>76973</t>
         </is>
@@ -23188,7 +23218,7 @@
           <t>VILARRUBLA Nuria</t>
         </is>
       </c>
-      <c r="U393" t="inlineStr">
+      <c r="X393" t="inlineStr">
         <is>
           <t>35746</t>
         </is>
@@ -23246,7 +23276,7 @@
           <t>DORIA VILARRUBLA Monica</t>
         </is>
       </c>
-      <c r="U394" t="inlineStr">
+      <c r="X394" t="inlineStr">
         <is>
           <t>53051</t>
         </is>
@@ -23304,7 +23334,7 @@
           <t>DELASSUS Marjorie</t>
         </is>
       </c>
-      <c r="U395" t="inlineStr">
+      <c r="X395" t="inlineStr">
         <is>
           <t>71964</t>
         </is>
@@ -23362,7 +23392,7 @@
           <t>SKACHOVA Monika</t>
         </is>
       </c>
-      <c r="U396" t="inlineStr">
+      <c r="X396" t="inlineStr">
         <is>
           <t>53078</t>
         </is>
@@ -23420,7 +23450,7 @@
           <t>WOLFFHARDT Viktoria</t>
         </is>
       </c>
-      <c r="U397" t="inlineStr">
+      <c r="X397" t="inlineStr">
         <is>
           <t>35303</t>
         </is>
@@ -23478,7 +23508,7 @@
           <t>FORROW Bethan</t>
         </is>
       </c>
-      <c r="U398" t="inlineStr">
+      <c r="X398" t="inlineStr">
         <is>
           <t>69065</t>
         </is>
@@ -23536,7 +23566,7 @@
           <t>MICOZZI Elena</t>
         </is>
       </c>
-      <c r="U399" t="inlineStr">
+      <c r="X399" t="inlineStr">
         <is>
           <t>84644</t>
         </is>
@@ -23594,7 +23624,7 @@
           <t>CHEN Shi</t>
         </is>
       </c>
-      <c r="U400" t="inlineStr">
+      <c r="X400" t="inlineStr">
         <is>
           <t>52027</t>
         </is>
@@ -23652,7 +23682,7 @@
           <t>OLAZABAL Klara</t>
         </is>
       </c>
-      <c r="U401" t="inlineStr">
+      <c r="X401" t="inlineStr">
         <is>
           <t>43985</t>
         </is>
@@ -23710,7 +23740,7 @@
           <t>LEIBFARTH Evy</t>
         </is>
       </c>
-      <c r="U402" t="inlineStr">
+      <c r="X402" t="inlineStr">
         <is>
           <t>83538</t>
         </is>
@@ -23768,7 +23798,7 @@
           <t>MILLER Ellis</t>
         </is>
       </c>
-      <c r="U403" t="inlineStr">
+      <c r="X403" t="inlineStr">
         <is>
           <t>75828</t>
         </is>
@@ -23826,7 +23856,7 @@
           <t>BAUDU Lucie</t>
         </is>
       </c>
-      <c r="U404" t="inlineStr">
+      <c r="X404" t="inlineStr">
         <is>
           <t>35669</t>
         </is>
@@ -23884,7 +23914,7 @@
           <t>ECKHARDT Kate</t>
         </is>
       </c>
-      <c r="U405" t="inlineStr">
+      <c r="X405" t="inlineStr">
         <is>
           <t>44815</t>
         </is>
@@ -23942,7 +23972,7 @@
           <t>DONNELLY Sage</t>
         </is>
       </c>
-      <c r="U406" t="inlineStr">
+      <c r="X406" t="inlineStr">
         <is>
           <t>60119</t>
         </is>
@@ -24000,7 +24030,7 @@
           <t>BERTONCELLI Marta</t>
         </is>
       </c>
-      <c r="U407" t="inlineStr">
+      <c r="X407" t="inlineStr">
         <is>
           <t>71982</t>
         </is>
@@ -24058,7 +24088,7 @@
           <t>HOCEVAR Eva Alina</t>
         </is>
       </c>
-      <c r="U408" t="inlineStr">
+      <c r="X408" t="inlineStr">
         <is>
           <t>75533</t>
         </is>
@@ -24116,7 +24146,7 @@
           <t>RIHOVA Eva</t>
         </is>
       </c>
-      <c r="U409" t="inlineStr">
+      <c r="X409" t="inlineStr">
         <is>
           <t>51791</t>
         </is>
@@ -24174,7 +24204,7 @@
           <t>FOX Noemie</t>
         </is>
       </c>
-      <c r="U410" t="inlineStr">
+      <c r="X410" t="inlineStr">
         <is>
           <t>44812</t>
         </is>
@@ -24232,7 +24262,7 @@
           <t>SCHORNBERG Jasmin</t>
         </is>
       </c>
-      <c r="U411" t="inlineStr">
+      <c r="X411" t="inlineStr">
         <is>
           <t>35206</t>
         </is>
@@ -24290,7 +24320,7 @@
           <t>BREGAZZI Ella</t>
         </is>
       </c>
-      <c r="U412" t="inlineStr">
+      <c r="X412" t="inlineStr">
         <is>
           <t>41598</t>
         </is>
@@ -24348,7 +24378,7 @@
           <t>APEL Elena</t>
         </is>
       </c>
-      <c r="U413" t="inlineStr">
+      <c r="X413" t="inlineStr">
         <is>
           <t>51837</t>
         </is>
@@ -24406,7 +24436,7 @@
           <t>SATILA Ana</t>
         </is>
       </c>
-      <c r="U414" t="inlineStr">
+      <c r="X414" t="inlineStr">
         <is>
           <t>35327</t>
         </is>
@@ -24464,7 +24494,7 @@
           <t>FISEROVA Tereza</t>
         </is>
       </c>
-      <c r="U415" t="inlineStr">
+      <c r="X415" t="inlineStr">
         <is>
           <t>42016</t>
         </is>
@@ -24522,7 +24552,7 @@
           <t>WERATSCHNIG Nadine</t>
         </is>
       </c>
-      <c r="U416" t="inlineStr">
+      <c r="X416" t="inlineStr">
         <is>
           <t>41613</t>
         </is>
@@ -24580,7 +24610,7 @@
           <t>HERZOG Andrea</t>
         </is>
       </c>
-      <c r="U417" t="inlineStr">
+      <c r="X417" t="inlineStr">
         <is>
           <t>55099</t>
         </is>
@@ -24638,7 +24668,7 @@
           <t>FOX Jessica</t>
         </is>
       </c>
-      <c r="U418" t="inlineStr">
+      <c r="X418" t="inlineStr">
         <is>
           <t>36526</t>
         </is>
@@ -24696,7 +24726,7 @@
           <t>SWETNAM Huw</t>
         </is>
       </c>
-      <c r="U419" t="inlineStr">
+      <c r="X419" t="inlineStr">
         <is>
           <t>35652</t>
         </is>
@@ -24754,7 +24784,7 @@
           <t>DE COSTER Gabriel</t>
         </is>
       </c>
-      <c r="U420" t="inlineStr">
+      <c r="X420" t="inlineStr">
         <is>
           <t>68818</t>
         </is>
@@ -24812,7 +24842,7 @@
           <t>DESNOS Mathieu</t>
         </is>
       </c>
-      <c r="U421" t="inlineStr">
+      <c r="X421" t="inlineStr">
         <is>
           <t>93791</t>
         </is>
@@ -24870,7 +24900,7 @@
           <t>PASIUT Michal</t>
         </is>
       </c>
-      <c r="U422" t="inlineStr">
+      <c r="X422" t="inlineStr">
         <is>
           <t>35095</t>
         </is>
@@ -24928,7 +24958,7 @@
           <t>LEITNER Mario</t>
         </is>
       </c>
-      <c r="U423" t="inlineStr">
+      <c r="X423" t="inlineStr">
         <is>
           <t>35546</t>
         </is>
@@ -24986,7 +25016,7 @@
           <t>SCHWEIKERT Fabian</t>
         </is>
       </c>
-      <c r="U424" t="inlineStr">
+      <c r="X424" t="inlineStr">
         <is>
           <t>38412</t>
         </is>
@@ -25044,7 +25074,7 @@
           <t>TESTEN Niko</t>
         </is>
       </c>
-      <c r="U425" t="inlineStr">
+      <c r="X425" t="inlineStr">
         <is>
           <t>39980</t>
         </is>
@@ -25102,7 +25132,7 @@
           <t>LLORENTE David</t>
         </is>
       </c>
-      <c r="U426" t="inlineStr">
+      <c r="X426" t="inlineStr">
         <is>
           <t>51850</t>
         </is>
@@ -25160,7 +25190,7 @@
           <t>GRIGAR Jakub</t>
         </is>
       </c>
-      <c r="U427" t="inlineStr">
+      <c r="X427" t="inlineStr">
         <is>
           <t>37284</t>
         </is>
@@ -25218,7 +25248,7 @@
           <t>NEVEU Boris</t>
         </is>
       </c>
-      <c r="U428" t="inlineStr">
+      <c r="X428" t="inlineStr">
         <is>
           <t>35396</t>
         </is>
@@ -25276,7 +25306,7 @@
           <t>THOMPSON Angus</t>
         </is>
       </c>
-      <c r="U429" t="inlineStr">
+      <c r="X429" t="inlineStr">
         <is>
           <t>44814</t>
         </is>
@@ -25334,7 +25364,7 @@
           <t>BEDA Marcello</t>
         </is>
       </c>
-      <c r="U430" t="inlineStr">
+      <c r="X430" t="inlineStr">
         <is>
           <t>39899</t>
         </is>
@@ -25392,7 +25422,7 @@
           <t>DELASSUS Anatole</t>
         </is>
       </c>
-      <c r="U431" t="inlineStr">
+      <c r="X431" t="inlineStr">
         <is>
           <t>84109</t>
         </is>
@@ -25450,7 +25480,7 @@
           <t>KARLSSON Max</t>
         </is>
       </c>
-      <c r="U432" t="inlineStr">
+      <c r="X432" t="inlineStr">
         <is>
           <t>35111</t>
         </is>
@@ -25508,7 +25538,7 @@
           <t>WERRO Lukas</t>
         </is>
       </c>
-      <c r="U433" t="inlineStr">
+      <c r="X433" t="inlineStr">
         <is>
           <t>35347</t>
         </is>
@@ -25566,7 +25596,7 @@
           <t>HALCIN Martin</t>
         </is>
       </c>
-      <c r="U434" t="inlineStr">
+      <c r="X434" t="inlineStr">
         <is>
           <t>35355</t>
         </is>
@@ -25624,7 +25654,7 @@
           <t>WAHLEN Fredrik</t>
         </is>
       </c>
-      <c r="U435" t="inlineStr">
+      <c r="X435" t="inlineStr">
         <is>
           <t>35102</t>
         </is>
@@ -25682,7 +25712,7 @@
           <t>QUAN Xin</t>
         </is>
       </c>
-      <c r="U436" t="inlineStr">
+      <c r="X436" t="inlineStr">
         <is>
           <t>62343</t>
         </is>
@@ -25740,7 +25770,7 @@
           <t>SRABOTNIK Martin</t>
         </is>
       </c>
-      <c r="U437" t="inlineStr">
+      <c r="X437" t="inlineStr">
         <is>
           <t>39080</t>
         </is>
@@ -25798,7 +25828,7 @@
           <t>GILBERT Callum</t>
         </is>
       </c>
-      <c r="U438" t="inlineStr">
+      <c r="X438" t="inlineStr">
         <is>
           <t>42090</t>
         </is>
@@ -25856,7 +25886,7 @@
           <t>MAJERCZAK Krzysztof</t>
         </is>
       </c>
-      <c r="U439" t="inlineStr">
+      <c r="X439" t="inlineStr">
         <is>
           <t>53647</t>
         </is>
@@ -25914,7 +25944,7 @@
           <t>OHRSTROM Isak</t>
         </is>
       </c>
-      <c r="U440" t="inlineStr">
+      <c r="X440" t="inlineStr">
         <is>
           <t>35101</t>
         </is>
@@ -25972,7 +26002,7 @@
           <t>MAXEINER Tim</t>
         </is>
       </c>
-      <c r="U441" t="inlineStr">
+      <c r="X441" t="inlineStr">
         <is>
           <t>35117</t>
         </is>
@@ -26030,7 +26060,7 @@
           <t>CRESPO Joan</t>
         </is>
       </c>
-      <c r="U442" t="inlineStr">
+      <c r="X442" t="inlineStr">
         <is>
           <t>35749</t>
         </is>
@@ -26088,7 +26118,7 @@
           <t>DOUGOUD Martin</t>
         </is>
       </c>
-      <c r="U443" t="inlineStr">
+      <c r="X443" t="inlineStr">
         <is>
           <t>35426</t>
         </is>
@@ -26146,7 +26176,7 @@
           <t>HRADILEK Vavrinec</t>
         </is>
       </c>
-      <c r="U444" t="inlineStr">
+      <c r="X444" t="inlineStr">
         <is>
           <t>35031</t>
         </is>
@@ -26204,7 +26234,7 @@
           <t>LAUNAY Antoine</t>
         </is>
       </c>
-      <c r="U445" t="inlineStr">
+      <c r="X445" t="inlineStr">
         <is>
           <t>68776</t>
         </is>
@@ -26262,7 +26292,7 @@
           <t>POPE Benjamin</t>
         </is>
       </c>
-      <c r="U446" t="inlineStr">
+      <c r="X446" t="inlineStr">
         <is>
           <t>51753</t>
         </is>
@@ -26320,7 +26350,7 @@
           <t>POPIELA Dariusz</t>
         </is>
       </c>
-      <c r="U447" t="inlineStr">
+      <c r="X447" t="inlineStr">
         <is>
           <t>35096</t>
         </is>
@@ -26378,7 +26408,7 @@
           <t>OSCHMAUTZ Felix</t>
         </is>
       </c>
-      <c r="U448" t="inlineStr">
+      <c r="X448" t="inlineStr">
         <is>
           <t>51856</t>
         </is>
@@ -26436,7 +26466,7 @@
           <t>BURGI Quentin</t>
         </is>
       </c>
-      <c r="U449" t="inlineStr">
+      <c r="X449" t="inlineStr">
         <is>
           <t>41590</t>
         </is>
@@ -26494,7 +26524,7 @@
           <t>IVALDI Zeno</t>
         </is>
       </c>
-      <c r="U450" t="inlineStr">
+      <c r="X450" t="inlineStr">
         <is>
           <t>35480</t>
         </is>
@@ -26552,7 +26582,7 @@
           <t>AIGNER Hannes</t>
         </is>
       </c>
-      <c r="U451" t="inlineStr">
+      <c r="X451" t="inlineStr">
         <is>
           <t>35115</t>
         </is>
@@ -26610,7 +26640,7 @@
           <t>DE GENNARO Giovanni</t>
         </is>
       </c>
-      <c r="U452" t="inlineStr">
+      <c r="X452" t="inlineStr">
         <is>
           <t>35244</t>
         </is>
@@ -26668,7 +26698,7 @@
           <t>KAUZER Peter</t>
         </is>
       </c>
-      <c r="U453" t="inlineStr">
+      <c r="X453" t="inlineStr">
         <is>
           <t>35589</t>
         </is>
@@ -26726,7 +26756,7 @@
           <t>HERNANZ Samuel</t>
         </is>
       </c>
-      <c r="U454" t="inlineStr">
+      <c r="X454" t="inlineStr">
         <is>
           <t>35786</t>
         </is>
@@ -26784,7 +26814,7 @@
           <t>PRINDIS Vit</t>
         </is>
       </c>
-      <c r="U455" t="inlineStr">
+      <c r="X455" t="inlineStr">
         <is>
           <t>35065</t>
         </is>
@@ -26842,7 +26872,7 @@
           <t>SMOLEN Michal</t>
         </is>
       </c>
-      <c r="U456" t="inlineStr">
+      <c r="X456" t="inlineStr">
         <is>
           <t>36397</t>
         </is>
@@ -26900,7 +26930,7 @@
           <t>DELFOUR Lucien</t>
         </is>
       </c>
-      <c r="U457" t="inlineStr">
+      <c r="X457" t="inlineStr">
         <is>
           <t>36537</t>
         </is>
@@ -26958,7 +26988,7 @@
           <t>PRSKAVEC Jiri</t>
         </is>
       </c>
-      <c r="U458" t="inlineStr">
+      <c r="X458" t="inlineStr">
         <is>
           <t>35033</t>
         </is>
@@ -27026,7 +27056,7 @@
           <t>ECKHARDT Kate</t>
         </is>
       </c>
-      <c r="U459" t="inlineStr">
+      <c r="X459" t="inlineStr">
         <is>
           <t>44815</t>
         </is>
@@ -27094,7 +27124,7 @@
           <t>HOCEVAR Eva Alina</t>
         </is>
       </c>
-      <c r="U460" t="inlineStr">
+      <c r="X460" t="inlineStr">
         <is>
           <t>75533</t>
         </is>
@@ -27162,7 +27192,7 @@
           <t>OLAZABAL Klara</t>
         </is>
       </c>
-      <c r="U461" t="inlineStr">
+      <c r="X461" t="inlineStr">
         <is>
           <t>43985</t>
         </is>
@@ -27230,7 +27260,7 @@
           <t>SATILA Ana</t>
         </is>
       </c>
-      <c r="U462" t="inlineStr">
+      <c r="X462" t="inlineStr">
         <is>
           <t>35327</t>
         </is>
@@ -27298,7 +27328,7 @@
           <t>SCHORNBERG Jasmin</t>
         </is>
       </c>
-      <c r="U463" t="inlineStr">
+      <c r="X463" t="inlineStr">
         <is>
           <t>35206</t>
         </is>
@@ -27366,7 +27396,7 @@
           <t>VILARRUBLA Nuria</t>
         </is>
       </c>
-      <c r="U464" t="inlineStr">
+      <c r="X464" t="inlineStr">
         <is>
           <t>35746</t>
         </is>
@@ -27434,7 +27464,7 @@
           <t>FISEROVA Tereza</t>
         </is>
       </c>
-      <c r="U465" t="inlineStr">
+      <c r="X465" t="inlineStr">
         <is>
           <t>42016</t>
         </is>
@@ -27502,7 +27532,7 @@
           <t>FOX Jessica</t>
         </is>
       </c>
-      <c r="U466" t="inlineStr">
+      <c r="X466" t="inlineStr">
         <is>
           <t>36526</t>
         </is>
@@ -27570,7 +27600,7 @@
           <t>HERZOG Andrea</t>
         </is>
       </c>
-      <c r="U467" t="inlineStr">
+      <c r="X467" t="inlineStr">
         <is>
           <t>55099</t>
         </is>
@@ -27638,7 +27668,7 @@
           <t>WERATSCHNIG Nadine</t>
         </is>
       </c>
-      <c r="U468" t="inlineStr">
+      <c r="X468" t="inlineStr">
         <is>
           <t>41613</t>
         </is>
@@ -27706,7 +27736,7 @@
           <t>DE GENNARO Giovanni</t>
         </is>
       </c>
-      <c r="U469" t="inlineStr">
+      <c r="X469" t="inlineStr">
         <is>
           <t>35244</t>
         </is>
@@ -27774,7 +27804,7 @@
           <t>AIGNER Hannes</t>
         </is>
       </c>
-      <c r="U470" t="inlineStr">
+      <c r="X470" t="inlineStr">
         <is>
           <t>35115</t>
         </is>
@@ -27842,7 +27872,7 @@
           <t>HALCIN Martin</t>
         </is>
       </c>
-      <c r="U471" t="inlineStr">
+      <c r="X471" t="inlineStr">
         <is>
           <t>35355</t>
         </is>
@@ -27910,7 +27940,7 @@
           <t>PRINDIS Vit</t>
         </is>
       </c>
-      <c r="U472" t="inlineStr">
+      <c r="X472" t="inlineStr">
         <is>
           <t>35065</t>
         </is>
@@ -27978,7 +28008,7 @@
           <t>HRADILEK Vavrinec</t>
         </is>
       </c>
-      <c r="U473" t="inlineStr">
+      <c r="X473" t="inlineStr">
         <is>
           <t>35031</t>
         </is>
@@ -28046,7 +28076,7 @@
           <t>NEVEU Boris</t>
         </is>
       </c>
-      <c r="U474" t="inlineStr">
+      <c r="X474" t="inlineStr">
         <is>
           <t>35396</t>
         </is>
@@ -28114,7 +28144,7 @@
           <t>KAUZER Peter</t>
         </is>
       </c>
-      <c r="U475" t="inlineStr">
+      <c r="X475" t="inlineStr">
         <is>
           <t>35589</t>
         </is>
@@ -28182,7 +28212,7 @@
           <t>PRSKAVEC Jiri</t>
         </is>
       </c>
-      <c r="U476" t="inlineStr">
+      <c r="X476" t="inlineStr">
         <is>
           <t>35033</t>
         </is>
@@ -28250,7 +28280,7 @@
           <t>MAXEINER Tim</t>
         </is>
       </c>
-      <c r="U477" t="inlineStr">
+      <c r="X477" t="inlineStr">
         <is>
           <t>35117</t>
         </is>
@@ -28318,7 +28348,7 @@
           <t>DELFOUR Lucien</t>
         </is>
       </c>
-      <c r="U478" t="inlineStr">
+      <c r="X478" t="inlineStr">
         <is>
           <t>36537</t>
         </is>
@@ -28381,7 +28411,7 @@
           <t>CHAPPELL Etienne</t>
         </is>
       </c>
-      <c r="U479" t="inlineStr">
+      <c r="X479" t="inlineStr">
         <is>
           <t>75833</t>
         </is>
@@ -28444,7 +28474,7 @@
           <t>SMOLEN Michal</t>
         </is>
       </c>
-      <c r="U480" t="inlineStr">
+      <c r="X480" t="inlineStr">
         <is>
           <t>36397</t>
         </is>
@@ -28507,7 +28537,7 @@
           <t>ZAZIABLO Jaroslaw</t>
         </is>
       </c>
-      <c r="U481" t="inlineStr">
+      <c r="X481" t="inlineStr">
         <is>
           <t>75728</t>
         </is>
@@ -28570,7 +28600,7 @@
           <t>RAJNIAK Boris</t>
         </is>
       </c>
-      <c r="U482" t="inlineStr">
+      <c r="X482" t="inlineStr">
         <is>
           <t>37309</t>
         </is>
@@ -28633,7 +28663,7 @@
           <t>WAHLEN Fredrik</t>
         </is>
       </c>
-      <c r="U483" t="inlineStr">
+      <c r="X483" t="inlineStr">
         <is>
           <t>35102</t>
         </is>
@@ -28696,7 +28726,7 @@
           <t>WOS Michal</t>
         </is>
       </c>
-      <c r="U484" t="inlineStr">
+      <c r="X484" t="inlineStr">
         <is>
           <t>65063</t>
         </is>
@@ -28759,7 +28789,7 @@
           <t>YOSHIDA Taku</t>
         </is>
       </c>
-      <c r="U485" t="inlineStr">
+      <c r="X485" t="inlineStr">
         <is>
           <t>41611</t>
         </is>
@@ -28822,7 +28852,7 @@
           <t>KARLSSON Max</t>
         </is>
       </c>
-      <c r="U486" t="inlineStr">
+      <c r="X486" t="inlineStr">
         <is>
           <t>35111</t>
         </is>
@@ -28885,7 +28915,7 @@
           <t>LIPPKE Fredderik</t>
         </is>
       </c>
-      <c r="U487" t="inlineStr">
+      <c r="X487" t="inlineStr">
         <is>
           <t>93810</t>
         </is>
@@ -28948,7 +28978,7 @@
           <t>LONG Tren</t>
         </is>
       </c>
-      <c r="U488" t="inlineStr">
+      <c r="X488" t="inlineStr">
         <is>
           <t>57124</t>
         </is>
@@ -29011,7 +29041,7 @@
           <t>MCCREERY Alistair</t>
         </is>
       </c>
-      <c r="U489" t="inlineStr">
+      <c r="X489" t="inlineStr">
         <is>
           <t>60125</t>
         </is>
@@ -29074,7 +29104,7 @@
           <t>DE DIONIGI Christian</t>
         </is>
       </c>
-      <c r="U490" t="inlineStr">
+      <c r="X490" t="inlineStr">
         <is>
           <t>43188</t>
         </is>
@@ -29137,7 +29167,7 @@
           <t>SEUMEL Paul</t>
         </is>
       </c>
-      <c r="U491" t="inlineStr">
+      <c r="X491" t="inlineStr">
         <is>
           <t>62076</t>
         </is>
@@ -29200,7 +29230,7 @@
           <t>STANOVSKY Samuel</t>
         </is>
       </c>
-      <c r="U492" t="inlineStr">
+      <c r="X492" t="inlineStr">
         <is>
           <t>84121</t>
         </is>
@@ -29263,7 +29293,7 @@
           <t>BENZIEN Mandy</t>
         </is>
       </c>
-      <c r="U493" t="inlineStr">
+      <c r="X493" t="inlineStr">
         <is>
           <t>102620</t>
         </is>
@@ -29326,7 +29356,7 @@
           <t>DONNELLY Sage</t>
         </is>
       </c>
-      <c r="U494" t="inlineStr">
+      <c r="X494" t="inlineStr">
         <is>
           <t>60119</t>
         </is>
@@ -29389,7 +29419,7 @@
           <t>TROMPETER Caroline</t>
         </is>
       </c>
-      <c r="U495" t="inlineStr">
+      <c r="X495" t="inlineStr">
         <is>
           <t>39167</t>
         </is>
@@ -29452,7 +29482,7 @@
           <t>NEE Ashley</t>
         </is>
       </c>
-      <c r="U496" t="inlineStr">
+      <c r="X496" t="inlineStr">
         <is>
           <t>36363</t>
         </is>
@@ -29515,7 +29545,7 @@
           <t>SCHWANHOLT Ann-Kathrin</t>
         </is>
       </c>
-      <c r="U497" t="inlineStr">
+      <c r="X497" t="inlineStr">
         <is>
           <t>43473</t>
         </is>
@@ -29578,7 +29608,7 @@
           <t>CHAPPELL Etienne</t>
         </is>
       </c>
-      <c r="U498" t="inlineStr">
+      <c r="X498" t="inlineStr">
         <is>
           <t>75833</t>
         </is>
@@ -29641,7 +29671,7 @@
           <t>WAHLEN Fredrik</t>
         </is>
       </c>
-      <c r="U499" t="inlineStr">
+      <c r="X499" t="inlineStr">
         <is>
           <t>35102</t>
         </is>
@@ -29704,7 +29734,7 @@
           <t>YOSHIDA Taku</t>
         </is>
       </c>
-      <c r="U500" t="inlineStr">
+      <c r="X500" t="inlineStr">
         <is>
           <t>41611</t>
         </is>
@@ -29767,7 +29797,7 @@
           <t>ZAZIABLO Jaroslaw</t>
         </is>
       </c>
-      <c r="U501" t="inlineStr">
+      <c r="X501" t="inlineStr">
         <is>
           <t>75728</t>
         </is>
@@ -29830,7 +29860,7 @@
           <t>DE DIONIGI Christian</t>
         </is>
       </c>
-      <c r="U502" t="inlineStr">
+      <c r="X502" t="inlineStr">
         <is>
           <t>43188</t>
         </is>
@@ -29893,7 +29923,7 @@
           <t>KARLSSON Max</t>
         </is>
       </c>
-      <c r="U503" t="inlineStr">
+      <c r="X503" t="inlineStr">
         <is>
           <t>35111</t>
         </is>
@@ -29956,7 +29986,7 @@
           <t>LONG Tren</t>
         </is>
       </c>
-      <c r="U504" t="inlineStr">
+      <c r="X504" t="inlineStr">
         <is>
           <t>57124</t>
         </is>
@@ -30019,7 +30049,7 @@
           <t>STANOVSKY Samuel</t>
         </is>
       </c>
-      <c r="U505" t="inlineStr">
+      <c r="X505" t="inlineStr">
         <is>
           <t>84121</t>
         </is>
@@ -30092,7 +30122,7 @@
           <t>DONNELLY Sage</t>
         </is>
       </c>
-      <c r="U506" t="inlineStr">
+      <c r="X506" t="inlineStr">
         <is>
           <t>60119</t>
         </is>
@@ -30165,7 +30195,7 @@
           <t>NEE Ashley</t>
         </is>
       </c>
-      <c r="U507" t="inlineStr">
+      <c r="X507" t="inlineStr">
         <is>
           <t>36363</t>
         </is>
@@ -30228,7 +30258,7 @@
           <t>SCHWANHOLT Ann-Kathrin</t>
         </is>
       </c>
-      <c r="U508" t="inlineStr">
+      <c r="X508" t="inlineStr">
         <is>
           <t>43473</t>
         </is>
@@ -30301,7 +30331,7 @@
           <t>TROMPETER Caroline</t>
         </is>
       </c>
-      <c r="U509" t="inlineStr">
+      <c r="X509" t="inlineStr">
         <is>
           <t>39167</t>
         </is>
@@ -30374,7 +30404,7 @@
           <t>CHAPPELL Etienne</t>
         </is>
       </c>
-      <c r="U510" t="inlineStr">
+      <c r="X510" t="inlineStr">
         <is>
           <t>75833</t>
         </is>
@@ -30447,7 +30477,7 @@
           <t>KARLSSON Max</t>
         </is>
       </c>
-      <c r="U511" t="inlineStr">
+      <c r="X511" t="inlineStr">
         <is>
           <t>35111</t>
         </is>
@@ -30520,7 +30550,7 @@
           <t>LONG Tren</t>
         </is>
       </c>
-      <c r="U512" t="inlineStr">
+      <c r="X512" t="inlineStr">
         <is>
           <t>57124</t>
         </is>
@@ -30593,7 +30623,7 @@
           <t>WAHLEN Fredrik</t>
         </is>
       </c>
-      <c r="U513" t="inlineStr">
+      <c r="X513" t="inlineStr">
         <is>
           <t>35102</t>
         </is>
@@ -30651,7 +30681,7 @@
           <t>VILARRUBLA Nuria</t>
         </is>
       </c>
-      <c r="U514" t="inlineStr">
+      <c r="X514" t="inlineStr">
         <is>
           <t>35746</t>
         </is>
@@ -30714,7 +30744,7 @@
           <t>TROMPETER Caroline</t>
         </is>
       </c>
-      <c r="U515" t="inlineStr">
+      <c r="X515" t="inlineStr">
         <is>
           <t>39167</t>
         </is>
@@ -30777,7 +30807,7 @@
           <t>SCHWANHOLT Ann-Kathrin</t>
         </is>
       </c>
-      <c r="U516" t="inlineStr">
+      <c r="X516" t="inlineStr">
         <is>
           <t>43473</t>
         </is>
@@ -30840,7 +30870,7 @@
           <t>WEGMAN Martina</t>
         </is>
       </c>
-      <c r="U517" t="inlineStr">
+      <c r="X517" t="inlineStr">
         <is>
           <t>35345</t>
         </is>
@@ -30903,7 +30933,7 @@
           <t>NEE Ashley</t>
         </is>
       </c>
-      <c r="U518" t="inlineStr">
+      <c r="X518" t="inlineStr">
         <is>
           <t>36363</t>
         </is>
@@ -30966,7 +30996,7 @@
           <t>DONNELLY Sage</t>
         </is>
       </c>
-      <c r="U519" t="inlineStr">
+      <c r="X519" t="inlineStr">
         <is>
           <t>60119</t>
         </is>
@@ -31029,7 +31059,7 @@
           <t>BENZIEN Mandy</t>
         </is>
       </c>
-      <c r="U520" t="inlineStr">
+      <c r="X520" t="inlineStr">
         <is>
           <t>102620</t>
         </is>
@@ -31092,7 +31122,7 @@
           <t>WAHLEN Fredrik</t>
         </is>
       </c>
-      <c r="U521" t="inlineStr">
+      <c r="X521" t="inlineStr">
         <is>
           <t>35102</t>
         </is>
@@ -31155,7 +31185,7 @@
           <t>LONG Tren</t>
         </is>
       </c>
-      <c r="U522" t="inlineStr">
+      <c r="X522" t="inlineStr">
         <is>
           <t>57124</t>
         </is>
@@ -31218,7 +31248,7 @@
           <t>SMOLEN Michal</t>
         </is>
       </c>
-      <c r="U523" t="inlineStr">
+      <c r="X523" t="inlineStr">
         <is>
           <t>36397</t>
         </is>
@@ -31281,7 +31311,7 @@
           <t>RAJNIAK Boris</t>
         </is>
       </c>
-      <c r="U524" t="inlineStr">
+      <c r="X524" t="inlineStr">
         <is>
           <t>37309</t>
         </is>
@@ -31344,7 +31374,7 @@
           <t>WOS Michal</t>
         </is>
       </c>
-      <c r="U525" t="inlineStr">
+      <c r="X525" t="inlineStr">
         <is>
           <t>65063</t>
         </is>
@@ -31407,7 +31437,7 @@
           <t>CHAPPELL Etienne</t>
         </is>
       </c>
-      <c r="U526" t="inlineStr">
+      <c r="X526" t="inlineStr">
         <is>
           <t>75833</t>
         </is>
@@ -31470,7 +31500,7 @@
           <t>YOSHIDA Taku</t>
         </is>
       </c>
-      <c r="U527" t="inlineStr">
+      <c r="X527" t="inlineStr">
         <is>
           <t>41611</t>
         </is>
@@ -31533,7 +31563,7 @@
           <t>LIPPKE Fredderik</t>
         </is>
       </c>
-      <c r="U528" t="inlineStr">
+      <c r="X528" t="inlineStr">
         <is>
           <t>93810</t>
         </is>
@@ -31596,7 +31626,7 @@
           <t>SEUMEL Paul</t>
         </is>
       </c>
-      <c r="U529" t="inlineStr">
+      <c r="X529" t="inlineStr">
         <is>
           <t>62076</t>
         </is>
@@ -31659,7 +31689,7 @@
           <t>STANOVSKY Samuel</t>
         </is>
       </c>
-      <c r="U530" t="inlineStr">
+      <c r="X530" t="inlineStr">
         <is>
           <t>84121</t>
         </is>
@@ -31722,7 +31752,7 @@
           <t>ZAZIABLO Jaroslaw</t>
         </is>
       </c>
-      <c r="U531" t="inlineStr">
+      <c r="X531" t="inlineStr">
         <is>
           <t>75728</t>
         </is>
@@ -31785,7 +31815,7 @@
           <t>DE DIONIGI Christian</t>
         </is>
       </c>
-      <c r="U532" t="inlineStr">
+      <c r="X532" t="inlineStr">
         <is>
           <t>43188</t>
         </is>
@@ -31848,7 +31878,7 @@
           <t>MCCREERY Alistair</t>
         </is>
       </c>
-      <c r="U533" t="inlineStr">
+      <c r="X533" t="inlineStr">
         <is>
           <t>60125</t>
         </is>
@@ -31911,7 +31941,7 @@
           <t>KARLSSON Max</t>
         </is>
       </c>
-      <c r="U534" t="inlineStr">
+      <c r="X534" t="inlineStr">
         <is>
           <t>35111</t>
         </is>

</xml_diff>